<commit_message>
feat(pricing): image L2 fallback, tier-union compare, and deployable prices-api
Add official+AIGC+TokenHub cascade for image draft JSON, P7 tier-union in
compare hub (no silent tier drops), diff vs online, and P6/P8 governance docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pricing/output/trinity-pricing-image.xlsx
+++ b/pricing/output/trinity-pricing-image.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q50"/>
+  <dimension ref="A1:Q61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -476,10 +476,10 @@
         <v>$0.039/张</v>
       </c>
       <c r="G2" t="str">
-        <v>—</v>
+        <v>¥0.3/张</v>
       </c>
       <c r="H2" t="str">
-        <v>—</v>
+        <v>$0.039/张</v>
       </c>
       <c r="I2" t="str">
         <v>—</v>
@@ -494,7 +494,7 @@
         <v>—</v>
       </c>
       <c r="M2" t="str">
-        <v>—</v>
+        <v>✅</v>
       </c>
       <c r="N2" t="str">
         <v>—</v>
@@ -511,28 +511,28 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>gemini-3-image</v>
+        <v/>
       </c>
       <c r="B3" t="str">
-        <v>gg-3.0</v>
+        <v/>
       </c>
       <c r="C3" t="str">
-        <v>Gemini</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>Gemini</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F3" t="str">
-        <v>$0.134/张</v>
+        <v>—</v>
       </c>
       <c r="G3" t="str">
-        <v>¥1/张</v>
+        <v>¥0.38/张</v>
       </c>
       <c r="H3" t="str">
-        <v>$0.135/张</v>
+        <v>$0.051/张</v>
       </c>
       <c r="I3" t="str">
         <v>—</v>
@@ -541,13 +541,13 @@
         <v>—</v>
       </c>
       <c r="K3" t="str">
-        <v>$0.137931/张</v>
+        <v>$0.0586/张</v>
       </c>
       <c r="L3" t="str">
         <v>—</v>
       </c>
       <c r="M3" t="str">
-        <v>⚠+0.7%</v>
+        <v>—</v>
       </c>
       <c r="N3" t="str">
         <v>—</v>
@@ -556,10 +556,10 @@
         <v>—</v>
       </c>
       <c r="P3" t="str">
-        <v>价⚠+2.9%</v>
+        <v>ℹ 官方无档 · 价⚠+14.9%</v>
       </c>
       <c r="Q3" t="str">
-        <v>API ID gemini-3-pro-image · Nano Banana Pro</v>
+        <v>API ID gemini-2.5-flash-image · Nano Banana</v>
       </c>
     </row>
     <row r="4">
@@ -576,16 +576,16 @@
         <v/>
       </c>
       <c r="E4" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F4" t="str">
-        <v>$0.134/张</v>
+        <v>—</v>
       </c>
       <c r="G4" t="str">
-        <v>¥1/张</v>
+        <v>¥0.46/张</v>
       </c>
       <c r="H4" t="str">
-        <v>$0.135/张</v>
+        <v>$0.063/张</v>
       </c>
       <c r="I4" t="str">
         <v>—</v>
@@ -594,13 +594,13 @@
         <v>—</v>
       </c>
       <c r="K4" t="str">
-        <v>$0.248276/张</v>
+        <v>$0.0635/张</v>
       </c>
       <c r="L4" t="str">
         <v>—</v>
       </c>
       <c r="M4" t="str">
-        <v>⚠+0.7%</v>
+        <v>—</v>
       </c>
       <c r="N4" t="str">
         <v>—</v>
@@ -609,36 +609,36 @@
         <v>—</v>
       </c>
       <c r="P4" t="str">
-        <v>🔍待核验 价⚠+85.3%</v>
+        <v>ℹ 官方无档 · 价⚠+0.8%</v>
       </c>
       <c r="Q4" t="str">
-        <v>API ID gemini-3-pro-image · Nano Banana Pro</v>
+        <v>API ID gemini-2.5-flash-image · Nano Banana</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v/>
+        <v>gemini-3-image</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>gg-3.0</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>Gemini</v>
       </c>
       <c r="D5" t="str">
-        <v/>
+        <v>Gemini</v>
       </c>
       <c r="E5" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F5" t="str">
-        <v>$0.24/张</v>
+        <v>$0.134/张</v>
       </c>
       <c r="G5" t="str">
-        <v>¥1.8/张</v>
+        <v>¥1/张</v>
       </c>
       <c r="H5" t="str">
-        <v>$0.24/张</v>
+        <v>$0.135/张</v>
       </c>
       <c r="I5" t="str">
         <v>—</v>
@@ -647,13 +647,13 @@
         <v>—</v>
       </c>
       <c r="K5" t="str">
-        <v>—</v>
+        <v>$0.137931/张</v>
       </c>
       <c r="L5" t="str">
         <v>—</v>
       </c>
       <c r="M5" t="str">
-        <v>✅</v>
+        <v>⚠+0.7%</v>
       </c>
       <c r="N5" t="str">
         <v>—</v>
@@ -662,7 +662,7 @@
         <v>—</v>
       </c>
       <c r="P5" t="str">
-        <v>ℹ 线上无同档刊例</v>
+        <v>价⚠+2.9%</v>
       </c>
       <c r="Q5" t="str">
         <v>API ID gemini-3-pro-image · Nano Banana Pro</v>
@@ -670,28 +670,28 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>gemini-3.1-image</v>
+        <v/>
       </c>
       <c r="B6" t="str">
-        <v>gg-3.1</v>
+        <v/>
       </c>
       <c r="C6" t="str">
-        <v>Gemini</v>
+        <v/>
       </c>
       <c r="D6" t="str">
-        <v>Gemini</v>
+        <v/>
       </c>
       <c r="E6" t="str">
-        <v>1K以下</v>
+        <v>2K</v>
       </c>
       <c r="F6" t="str">
-        <v>$0.045/张</v>
+        <v>$0.134/张</v>
       </c>
       <c r="G6" t="str">
-        <v>¥0.333/张</v>
+        <v>¥1/张</v>
       </c>
       <c r="H6" t="str">
-        <v>$0.045/张</v>
+        <v>$0.135/张</v>
       </c>
       <c r="I6" t="str">
         <v>—</v>
@@ -700,13 +700,13 @@
         <v>—</v>
       </c>
       <c r="K6" t="str">
-        <v>—</v>
+        <v>$0.248276/张</v>
       </c>
       <c r="L6" t="str">
         <v>—</v>
       </c>
       <c r="M6" t="str">
-        <v>✅</v>
+        <v>⚠+0.7%</v>
       </c>
       <c r="N6" t="str">
         <v>—</v>
@@ -715,10 +715,10 @@
         <v>—</v>
       </c>
       <c r="P6" t="str">
-        <v>ℹ 线上无同档刊例</v>
+        <v>🔍待核验 价⚠+85.3%</v>
       </c>
       <c r="Q6" t="str">
-        <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
+        <v>API ID gemini-3-pro-image · Nano Banana Pro</v>
       </c>
     </row>
     <row r="7">
@@ -735,16 +735,16 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>1K</v>
+        <v>4K</v>
       </c>
       <c r="F7" t="str">
-        <v>$0.067/张</v>
+        <v>$0.24/张</v>
       </c>
       <c r="G7" t="str">
-        <v>¥0.5/张</v>
+        <v>¥1.8/张</v>
       </c>
       <c r="H7" t="str">
-        <v>$0.067/张</v>
+        <v>$0.24/张</v>
       </c>
       <c r="I7" t="str">
         <v>—</v>
@@ -753,7 +753,7 @@
         <v>—</v>
       </c>
       <c r="K7" t="str">
-        <v>$0.077/张</v>
+        <v>—</v>
       </c>
       <c r="L7" t="str">
         <v>—</v>
@@ -768,36 +768,36 @@
         <v>—</v>
       </c>
       <c r="P7" t="str">
-        <v>价⚠+14.9%</v>
+        <v>ℹ 线上无同档刊例</v>
       </c>
       <c r="Q7" t="str">
-        <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
+        <v>API ID gemini-3-pro-image · Nano Banana Pro</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>gemini-3.1-image</v>
       </c>
       <c r="B8" t="str">
-        <v/>
+        <v>gg-3.1</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>Gemini</v>
       </c>
       <c r="D8" t="str">
-        <v/>
+        <v>Gemini</v>
       </c>
       <c r="E8" t="str">
-        <v>2K</v>
+        <v>1K以下</v>
       </c>
       <c r="F8" t="str">
-        <v>$0.101/张</v>
+        <v>$0.045/张</v>
       </c>
       <c r="G8" t="str">
-        <v>¥0.75/张</v>
+        <v>¥0.333/张</v>
       </c>
       <c r="H8" t="str">
-        <v>$0.101/张</v>
+        <v>$0.045/张</v>
       </c>
       <c r="I8" t="str">
         <v>—</v>
@@ -806,7 +806,7 @@
         <v>—</v>
       </c>
       <c r="K8" t="str">
-        <v>$0.1154/张</v>
+        <v>$0.0513/张</v>
       </c>
       <c r="L8" t="str">
         <v>—</v>
@@ -821,7 +821,7 @@
         <v>—</v>
       </c>
       <c r="P8" t="str">
-        <v>价⚠+14.3%</v>
+        <v>价⚠+14%</v>
       </c>
       <c r="Q8" t="str">
         <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
@@ -841,16 +841,16 @@
         <v/>
       </c>
       <c r="E9" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F9" t="str">
-        <v>$0.151/张</v>
+        <v>$0.067/张</v>
       </c>
       <c r="G9" t="str">
-        <v>¥1.12/张</v>
+        <v>¥0.5/张</v>
       </c>
       <c r="H9" t="str">
-        <v>$0.151/张</v>
+        <v>$0.067/张</v>
       </c>
       <c r="I9" t="str">
         <v>—</v>
@@ -859,7 +859,7 @@
         <v>—</v>
       </c>
       <c r="K9" t="str">
-        <v>$0.154483/张</v>
+        <v>$0.077/张</v>
       </c>
       <c r="L9" t="str">
         <v>—</v>
@@ -874,7 +874,7 @@
         <v>—</v>
       </c>
       <c r="P9" t="str">
-        <v>价⚠+2.3%</v>
+        <v>价⚠+14.9%</v>
       </c>
       <c r="Q9" t="str">
         <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
@@ -882,28 +882,28 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>midjourney-v7</v>
+        <v/>
       </c>
       <c r="B10" t="str">
-        <v>mj-v7</v>
+        <v/>
       </c>
       <c r="C10" t="str">
-        <v>Midjourney</v>
+        <v/>
       </c>
       <c r="D10" t="str">
-        <v>Midjourney</v>
+        <v/>
       </c>
       <c r="E10" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F10" t="str">
-        <v>$0.039/张</v>
+        <v>$0.101/张</v>
       </c>
       <c r="G10" t="str">
-        <v>—</v>
+        <v>¥0.75/张</v>
       </c>
       <c r="H10" t="str">
-        <v>—</v>
+        <v>$0.101/张</v>
       </c>
       <c r="I10" t="str">
         <v>—</v>
@@ -912,13 +912,13 @@
         <v>—</v>
       </c>
       <c r="K10" t="str">
-        <v>$0.0462/张</v>
+        <v>$0.1154/张</v>
       </c>
       <c r="L10" t="str">
         <v>—</v>
       </c>
       <c r="M10" t="str">
-        <v>—</v>
+        <v>✅</v>
       </c>
       <c r="N10" t="str">
         <v>—</v>
@@ -927,36 +927,36 @@
         <v>—</v>
       </c>
       <c r="P10" t="str">
-        <v>价⚠+18.5%</v>
+        <v>价⚠+14.3%</v>
       </c>
       <c r="Q10" t="str">
-        <v>订阅制，无公开 API 按张价目</v>
+        <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>openai-image2-high</v>
+        <v/>
       </c>
       <c r="B11" t="str">
-        <v>og-image2-high</v>
+        <v/>
       </c>
       <c r="C11" t="str">
-        <v>OpenAI</v>
+        <v/>
       </c>
       <c r="D11" t="str">
-        <v>OpenAI</v>
+        <v/>
       </c>
       <c r="E11" t="str">
-        <v>1K</v>
+        <v>4K</v>
       </c>
       <c r="F11" t="str">
-        <v>$0.211/张</v>
+        <v>$0.151/张</v>
       </c>
       <c r="G11" t="str">
-        <v>¥1.583/张</v>
+        <v>¥1.12/张</v>
       </c>
       <c r="H11" t="str">
-        <v>$0.211/张</v>
+        <v>$0.151/张</v>
       </c>
       <c r="I11" t="str">
         <v>—</v>
@@ -965,7 +965,7 @@
         <v>—</v>
       </c>
       <c r="K11" t="str">
-        <v>$1.583/张</v>
+        <v>$0.154483/张</v>
       </c>
       <c r="L11" t="str">
         <v>—</v>
@@ -980,10 +980,10 @@
         <v>—</v>
       </c>
       <c r="P11" t="str">
-        <v>🔍待核验 价⚠+650.2%</v>
+        <v>价⚠+2.3%</v>
       </c>
       <c r="Q11" t="str">
-        <v/>
+        <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
       </c>
     </row>
     <row r="12">
@@ -1000,16 +1000,16 @@
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>2K</v>
+        <v>1K以下</v>
       </c>
       <c r="F12" t="str">
-        <v>$0.428/张</v>
+        <v>—</v>
       </c>
       <c r="G12" t="str">
-        <v>¥3.21/张</v>
+        <v>—</v>
       </c>
       <c r="H12" t="str">
-        <v>$0.428/张</v>
+        <v>—</v>
       </c>
       <c r="I12" t="str">
         <v>—</v>
@@ -1018,13 +1018,13 @@
         <v>—</v>
       </c>
       <c r="K12" t="str">
-        <v>$3.21/张</v>
+        <v>$0.0513/张</v>
       </c>
       <c r="L12" t="str">
         <v>—</v>
       </c>
       <c r="M12" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N12" t="str">
         <v>—</v>
@@ -1033,36 +1033,36 @@
         <v>—</v>
       </c>
       <c r="P12" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>—</v>
       </c>
       <c r="Q12" t="str">
-        <v/>
+        <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v/>
+        <v>midjourney-v7</v>
       </c>
       <c r="B13" t="str">
-        <v/>
+        <v>mj-v7</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>Midjourney</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>Midjourney</v>
       </c>
       <c r="E13" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F13" t="str">
-        <v>$0.712/张</v>
+        <v>$0.039/张</v>
       </c>
       <c r="G13" t="str">
-        <v>¥5.34/张</v>
+        <v>¥0.3/张</v>
       </c>
       <c r="H13" t="str">
-        <v>$0.712/张</v>
+        <v>$0.039/张</v>
       </c>
       <c r="I13" t="str">
         <v>—</v>
@@ -1071,7 +1071,7 @@
         <v>—</v>
       </c>
       <c r="K13" t="str">
-        <v>$5.34/张</v>
+        <v>$0.0462/张</v>
       </c>
       <c r="L13" t="str">
         <v>—</v>
@@ -1086,36 +1086,36 @@
         <v>—</v>
       </c>
       <c r="P13" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>价⚠+18.5%</v>
       </c>
       <c r="Q13" t="str">
-        <v/>
+        <v>订阅制，无公开 API 按张价目</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>openai-image2-low</v>
+        <v/>
       </c>
       <c r="B14" t="str">
-        <v>og-image2-low</v>
+        <v/>
       </c>
       <c r="C14" t="str">
-        <v>OpenAI</v>
+        <v/>
       </c>
       <c r="D14" t="str">
-        <v>OpenAI</v>
+        <v/>
       </c>
       <c r="E14" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F14" t="str">
-        <v>$0.006/张</v>
+        <v>—</v>
       </c>
       <c r="G14" t="str">
-        <v>¥0.045/张</v>
+        <v>¥0.38/张</v>
       </c>
       <c r="H14" t="str">
-        <v>$0.006/张</v>
+        <v>$0.051/张</v>
       </c>
       <c r="I14" t="str">
         <v>—</v>
@@ -1124,13 +1124,13 @@
         <v>—</v>
       </c>
       <c r="K14" t="str">
-        <v>$0.045/张</v>
+        <v>$0.052414/张</v>
       </c>
       <c r="L14" t="str">
         <v>—</v>
       </c>
       <c r="M14" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N14" t="str">
         <v>—</v>
@@ -1139,10 +1139,10 @@
         <v>—</v>
       </c>
       <c r="P14" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>ℹ 官方无档 · 价⚠+2.8%</v>
       </c>
       <c r="Q14" t="str">
-        <v/>
+        <v>订阅制，无公开 API 按张价目</v>
       </c>
     </row>
     <row r="15">
@@ -1159,16 +1159,16 @@
         <v/>
       </c>
       <c r="E15" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F15" t="str">
-        <v>$0.012/张</v>
+        <v>—</v>
       </c>
       <c r="G15" t="str">
-        <v>¥0.09/张</v>
+        <v>¥0.46/张</v>
       </c>
       <c r="H15" t="str">
-        <v>$0.012/张</v>
+        <v>$0.063/张</v>
       </c>
       <c r="I15" t="str">
         <v>—</v>
@@ -1177,13 +1177,13 @@
         <v>—</v>
       </c>
       <c r="K15" t="str">
-        <v>$0.09/张</v>
+        <v>$0.063448/张</v>
       </c>
       <c r="L15" t="str">
         <v>—</v>
       </c>
       <c r="M15" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N15" t="str">
         <v>—</v>
@@ -1192,36 +1192,36 @@
         <v>—</v>
       </c>
       <c r="P15" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>ℹ 官方无档 · 价⚠+0.7%</v>
       </c>
       <c r="Q15" t="str">
-        <v/>
+        <v>订阅制，无公开 API 按张价目</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>openai-image2-high</v>
       </c>
       <c r="B16" t="str">
-        <v/>
+        <v>og-image2-high</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>OpenAI</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>OpenAI</v>
       </c>
       <c r="E16" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F16" t="str">
-        <v>$0.02/张</v>
+        <v>$0.211/张</v>
       </c>
       <c r="G16" t="str">
-        <v>¥0.15/张</v>
+        <v>¥1.583/张</v>
       </c>
       <c r="H16" t="str">
-        <v>$0.02/张</v>
+        <v>$0.211/张</v>
       </c>
       <c r="I16" t="str">
         <v>—</v>
@@ -1230,7 +1230,7 @@
         <v>—</v>
       </c>
       <c r="K16" t="str">
-        <v>$0.15/张</v>
+        <v>$1.583/张</v>
       </c>
       <c r="L16" t="str">
         <v>—</v>
@@ -1245,7 +1245,7 @@
         <v>—</v>
       </c>
       <c r="P16" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>🔍待核验 价⚠+650.2%</v>
       </c>
       <c r="Q16" t="str">
         <v/>
@@ -1253,28 +1253,28 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>openai-image2-medium</v>
+        <v/>
       </c>
       <c r="B17" t="str">
-        <v>og-image2-medium</v>
+        <v/>
       </c>
       <c r="C17" t="str">
-        <v>OpenAI</v>
+        <v/>
       </c>
       <c r="D17" t="str">
-        <v>OpenAI</v>
+        <v/>
       </c>
       <c r="E17" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F17" t="str">
-        <v>$0.053/张</v>
+        <v>$0.428/张</v>
       </c>
       <c r="G17" t="str">
-        <v>¥0.398/张</v>
+        <v>¥3.21/张</v>
       </c>
       <c r="H17" t="str">
-        <v>$0.053/张</v>
+        <v>$0.428/张</v>
       </c>
       <c r="I17" t="str">
         <v>—</v>
@@ -1283,7 +1283,7 @@
         <v>—</v>
       </c>
       <c r="K17" t="str">
-        <v>$0.398/张</v>
+        <v>$3.21/张</v>
       </c>
       <c r="L17" t="str">
         <v>—</v>
@@ -1298,7 +1298,7 @@
         <v>—</v>
       </c>
       <c r="P17" t="str">
-        <v>🔍待核验 价⚠+650.9%</v>
+        <v>🔍待核验 价⚠+650%</v>
       </c>
       <c r="Q17" t="str">
         <v/>
@@ -1318,16 +1318,16 @@
         <v/>
       </c>
       <c r="E18" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F18" t="str">
-        <v>$0.107/张</v>
+        <v>$0.712/张</v>
       </c>
       <c r="G18" t="str">
-        <v>¥0.803/张</v>
+        <v>¥5.34/张</v>
       </c>
       <c r="H18" t="str">
-        <v>$0.107/张</v>
+        <v>$0.712/张</v>
       </c>
       <c r="I18" t="str">
         <v>—</v>
@@ -1336,7 +1336,7 @@
         <v>—</v>
       </c>
       <c r="K18" t="str">
-        <v>$0.803/张</v>
+        <v>$5.34/张</v>
       </c>
       <c r="L18" t="str">
         <v>—</v>
@@ -1351,7 +1351,7 @@
         <v>—</v>
       </c>
       <c r="P18" t="str">
-        <v>🔍待核验 价⚠+650.5%</v>
+        <v>🔍待核验 价⚠+650%</v>
       </c>
       <c r="Q18" t="str">
         <v/>
@@ -1359,28 +1359,28 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v/>
+        <v>openai-image2-low</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>og-image2-low</v>
       </c>
       <c r="C19" t="str">
-        <v/>
+        <v>OpenAI</v>
       </c>
       <c r="D19" t="str">
-        <v/>
+        <v>OpenAI</v>
       </c>
       <c r="E19" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F19" t="str">
-        <v>$0.178/张</v>
+        <v>$0.006/张</v>
       </c>
       <c r="G19" t="str">
-        <v>¥1.335/张</v>
+        <v>¥0.045/张</v>
       </c>
       <c r="H19" t="str">
-        <v>$0.178/张</v>
+        <v>$0.006/张</v>
       </c>
       <c r="I19" t="str">
         <v>—</v>
@@ -1389,7 +1389,7 @@
         <v>—</v>
       </c>
       <c r="K19" t="str">
-        <v>$1.335/张</v>
+        <v>$0.045/张</v>
       </c>
       <c r="L19" t="str">
         <v>—</v>
@@ -1412,28 +1412,28 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>vidu-q2</v>
+        <v/>
       </c>
       <c r="B20" t="str">
-        <v>vidu-q2</v>
+        <v/>
       </c>
       <c r="C20" t="str">
-        <v>Vidu</v>
+        <v/>
       </c>
       <c r="D20" t="str">
-        <v>Vidu</v>
+        <v/>
       </c>
       <c r="E20" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F20" t="str">
-        <v>¥0.1875/张</v>
+        <v>$0.012/张</v>
       </c>
       <c r="G20" t="str">
-        <v>¥0.1875/张</v>
+        <v>¥0.09/张</v>
       </c>
       <c r="H20" t="str">
-        <v>$0.0288461538461539/张</v>
+        <v>$0.012/张</v>
       </c>
       <c r="I20" t="str">
         <v>—</v>
@@ -1442,10 +1442,10 @@
         <v>—</v>
       </c>
       <c r="K20" t="str">
-        <v>$0.0577/张</v>
+        <v>$0.09/张</v>
       </c>
       <c r="L20" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M20" t="str">
         <v>✅</v>
@@ -1457,10 +1457,10 @@
         <v>—</v>
       </c>
       <c r="P20" t="str">
-        <v>🔍待核验 价⚠+100%</v>
+        <v>🔍待核验 价⚠+650%</v>
       </c>
       <c r="Q20" t="str">
-        <v>viduq2 文生图 · 积分计价</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -1477,16 +1477,16 @@
         <v/>
       </c>
       <c r="E21" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F21" t="str">
-        <v>¥0.25/张</v>
+        <v>$0.02/张</v>
       </c>
       <c r="G21" t="str">
-        <v>¥0.25/张</v>
+        <v>¥0.15/张</v>
       </c>
       <c r="H21" t="str">
-        <v>$0.0384615384615385/张</v>
+        <v>$0.02/张</v>
       </c>
       <c r="I21" t="str">
         <v>—</v>
@@ -1495,10 +1495,10 @@
         <v>—</v>
       </c>
       <c r="K21" t="str">
-        <v>$0.077/张</v>
+        <v>$0.15/张</v>
       </c>
       <c r="L21" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M21" t="str">
         <v>✅</v>
@@ -1510,36 +1510,36 @@
         <v>—</v>
       </c>
       <c r="P21" t="str">
-        <v>🔍待核验 价⚠+100.2%</v>
+        <v>🔍待核验 价⚠+650%</v>
       </c>
       <c r="Q21" t="str">
-        <v>viduq2 文生图 · 积分计价</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v/>
+        <v>openai-image2-medium</v>
       </c>
       <c r="B22" t="str">
-        <v/>
+        <v>og-image2-medium</v>
       </c>
       <c r="C22" t="str">
-        <v/>
+        <v>OpenAI</v>
       </c>
       <c r="D22" t="str">
-        <v/>
+        <v>OpenAI</v>
       </c>
       <c r="E22" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F22" t="str">
-        <v>¥0.3125/张</v>
+        <v>$0.053/张</v>
       </c>
       <c r="G22" t="str">
-        <v>¥0.3125/张</v>
+        <v>¥0.398/张</v>
       </c>
       <c r="H22" t="str">
-        <v>$0.0480769230769231/张</v>
+        <v>$0.053/张</v>
       </c>
       <c r="I22" t="str">
         <v>—</v>
@@ -1548,10 +1548,10 @@
         <v>—</v>
       </c>
       <c r="K22" t="str">
-        <v>$0.0482/张</v>
+        <v>$0.398/张</v>
       </c>
       <c r="L22" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M22" t="str">
         <v>✅</v>
@@ -1563,36 +1563,36 @@
         <v>—</v>
       </c>
       <c r="P22" t="str">
-        <v>价✅</v>
+        <v>🔍待核验 价⚠+650.9%</v>
       </c>
       <c r="Q22" t="str">
-        <v>viduq2 文生图 · 积分计价</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>jimeng-4.0</v>
+        <v/>
       </c>
       <c r="B23" t="str">
-        <v>jimeng-4.0</v>
+        <v/>
       </c>
       <c r="C23" t="str">
-        <v>即梦</v>
+        <v/>
       </c>
       <c r="D23" t="str">
-        <v>即梦</v>
+        <v/>
       </c>
       <c r="E23" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F23" t="str">
-        <v>¥0.22/张</v>
+        <v>$0.107/张</v>
       </c>
       <c r="G23" t="str">
-        <v>¥0.22/张</v>
+        <v>¥0.803/张</v>
       </c>
       <c r="H23" t="str">
-        <v>$0.0339/张</v>
+        <v>$0.107/张</v>
       </c>
       <c r="I23" t="str">
         <v>—</v>
@@ -1601,10 +1601,10 @@
         <v>—</v>
       </c>
       <c r="K23" t="str">
-        <v>$0.0339/张</v>
+        <v>$0.803/张</v>
       </c>
       <c r="L23" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M23" t="str">
         <v>✅</v>
@@ -1616,7 +1616,7 @@
         <v>—</v>
       </c>
       <c r="P23" t="str">
-        <v>价✅</v>
+        <v>🔍待核验 价⚠+650.5%</v>
       </c>
       <c r="Q23" t="str">
         <v/>
@@ -1636,16 +1636,16 @@
         <v/>
       </c>
       <c r="E24" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F24" t="str">
-        <v>¥0.22/张</v>
+        <v>$0.178/张</v>
       </c>
       <c r="G24" t="str">
-        <v>¥0.22/张</v>
+        <v>¥1.335/张</v>
       </c>
       <c r="H24" t="str">
-        <v>$0.0339/张</v>
+        <v>$0.178/张</v>
       </c>
       <c r="I24" t="str">
         <v>—</v>
@@ -1654,10 +1654,10 @@
         <v>—</v>
       </c>
       <c r="K24" t="str">
-        <v>$0.0339/张</v>
+        <v>$1.335/张</v>
       </c>
       <c r="L24" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M24" t="str">
         <v>✅</v>
@@ -1669,7 +1669,7 @@
         <v>—</v>
       </c>
       <c r="P24" t="str">
-        <v>价✅</v>
+        <v>🔍待核验 价⚠+650%</v>
       </c>
       <c r="Q24" t="str">
         <v/>
@@ -1677,28 +1677,28 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v/>
+        <v>vidu-q2</v>
       </c>
       <c r="B25" t="str">
-        <v/>
+        <v>vidu-q2</v>
       </c>
       <c r="C25" t="str">
-        <v/>
+        <v>Vidu</v>
       </c>
       <c r="D25" t="str">
-        <v/>
+        <v>Vidu</v>
       </c>
       <c r="E25" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F25" t="str">
-        <v>¥0.22/张</v>
+        <v>¥0.1875/张</v>
       </c>
       <c r="G25" t="str">
-        <v>¥0.22/张</v>
+        <v>¥0.1875/张</v>
       </c>
       <c r="H25" t="str">
-        <v>$0.0339/张</v>
+        <v>$0.0288461538461539/张</v>
       </c>
       <c r="I25" t="str">
         <v>—</v>
@@ -1707,7 +1707,7 @@
         <v>—</v>
       </c>
       <c r="K25" t="str">
-        <v>$0.0339/张</v>
+        <v>$0.0577/张</v>
       </c>
       <c r="L25" t="str">
         <v>✅</v>
@@ -1722,36 +1722,36 @@
         <v>—</v>
       </c>
       <c r="P25" t="str">
-        <v>价✅</v>
+        <v>🔍待核验 价⚠+100%</v>
       </c>
       <c r="Q25" t="str">
-        <v/>
+        <v>viduq2 文生图 · 积分计价</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>kling-2.1</v>
+        <v/>
       </c>
       <c r="B26" t="str">
-        <v>kling-2.1</v>
+        <v/>
       </c>
       <c r="C26" t="str">
-        <v>可灵</v>
+        <v/>
       </c>
       <c r="D26" t="str">
-        <v>可灵</v>
+        <v/>
       </c>
       <c r="E26" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F26" t="str">
-        <v>¥0.1/张</v>
+        <v>¥0.25/张</v>
       </c>
       <c r="G26" t="str">
-        <v>¥0.1/张</v>
+        <v>¥0.25/张</v>
       </c>
       <c r="H26" t="str">
-        <v>$0.014/张</v>
+        <v>$0.0384615384615385/张</v>
       </c>
       <c r="I26" t="str">
         <v>—</v>
@@ -1760,13 +1760,13 @@
         <v>—</v>
       </c>
       <c r="K26" t="str">
-        <v>$0.013793/张</v>
+        <v>$0.077/张</v>
       </c>
       <c r="L26" t="str">
         <v>✅</v>
       </c>
       <c r="M26" t="str">
-        <v>⚠-9%</v>
+        <v>✅</v>
       </c>
       <c r="N26" t="str">
         <v>—</v>
@@ -1775,10 +1775,10 @@
         <v>—</v>
       </c>
       <c r="P26" t="str">
-        <v>价⚠-10.3%</v>
+        <v>🔍待核验 价⚠+100.2%</v>
       </c>
       <c r="Q26" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>viduq2 文生图 · 积分计价</v>
       </c>
     </row>
     <row r="27">
@@ -1795,16 +1795,16 @@
         <v/>
       </c>
       <c r="E27" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F27" t="str">
-        <v>¥0.1/张</v>
+        <v>¥0.3125/张</v>
       </c>
       <c r="G27" t="str">
-        <v>¥0.1/张</v>
+        <v>¥0.3125/张</v>
       </c>
       <c r="H27" t="str">
-        <v>$0.014/张</v>
+        <v>$0.0480769230769231/张</v>
       </c>
       <c r="I27" t="str">
         <v>—</v>
@@ -1813,13 +1813,13 @@
         <v>—</v>
       </c>
       <c r="K27" t="str">
-        <v>$0.077241/张</v>
+        <v>$0.0482/张</v>
       </c>
       <c r="L27" t="str">
         <v>✅</v>
       </c>
       <c r="M27" t="str">
-        <v>⚠-9%</v>
+        <v>✅</v>
       </c>
       <c r="N27" t="str">
         <v>—</v>
@@ -1828,36 +1828,36 @@
         <v>—</v>
       </c>
       <c r="P27" t="str">
-        <v>🔍待核验 价⚠+402.1%</v>
+        <v>价✅</v>
       </c>
       <c r="Q27" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v>viduq2 文生图 · 积分计价</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v/>
+        <v>jimeng-4.0</v>
       </c>
       <c r="B28" t="str">
-        <v/>
+        <v>jimeng-4.0</v>
       </c>
       <c r="C28" t="str">
-        <v/>
+        <v>即梦</v>
       </c>
       <c r="D28" t="str">
-        <v/>
+        <v>即梦</v>
       </c>
       <c r="E28" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F28" t="str">
-        <v>¥0.26/张</v>
+        <v>¥0.22/张</v>
       </c>
       <c r="G28" t="str">
-        <v>¥0.26/张</v>
+        <v>¥0.22/张</v>
       </c>
       <c r="H28" t="str">
-        <v>$0.037/张</v>
+        <v>$0.0339/张</v>
       </c>
       <c r="I28" t="str">
         <v>—</v>
@@ -1866,13 +1866,13 @@
         <v>—</v>
       </c>
       <c r="K28" t="str">
-        <v>—</v>
+        <v>$0.0339/张</v>
       </c>
       <c r="L28" t="str">
         <v>✅</v>
       </c>
       <c r="M28" t="str">
-        <v>⚠-7.5%</v>
+        <v>✅</v>
       </c>
       <c r="N28" t="str">
         <v>—</v>
@@ -1881,36 +1881,36 @@
         <v>—</v>
       </c>
       <c r="P28" t="str">
-        <v>ℹ 线上无同档刊例</v>
+        <v>价✅</v>
       </c>
       <c r="Q28" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>kling-3</v>
+        <v/>
       </c>
       <c r="B29" t="str">
-        <v>kling-3.0</v>
+        <v/>
       </c>
       <c r="C29" t="str">
-        <v>可灵</v>
+        <v/>
       </c>
       <c r="D29" t="str">
-        <v>可灵</v>
+        <v/>
       </c>
       <c r="E29" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F29" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.22/张</v>
       </c>
       <c r="G29" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.22/张</v>
       </c>
       <c r="H29" t="str">
-        <v>$0.028/张</v>
+        <v>$0.0339/张</v>
       </c>
       <c r="I29" t="str">
         <v>—</v>
@@ -1919,13 +1919,13 @@
         <v>—</v>
       </c>
       <c r="K29" t="str">
-        <v>$0.0308/张</v>
+        <v>$0.0339/张</v>
       </c>
       <c r="L29" t="str">
         <v>✅</v>
       </c>
       <c r="M29" t="str">
-        <v>⚠-9%</v>
+        <v>✅</v>
       </c>
       <c r="N29" t="str">
         <v>—</v>
@@ -1937,7 +1937,7 @@
         <v>价✅</v>
       </c>
       <c r="Q29" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1954,16 +1954,16 @@
         <v/>
       </c>
       <c r="E30" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F30" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.22/张</v>
       </c>
       <c r="G30" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.22/张</v>
       </c>
       <c r="H30" t="str">
-        <v>$0.028/张</v>
+        <v>$0.0339/张</v>
       </c>
       <c r="I30" t="str">
         <v>—</v>
@@ -1972,13 +1972,13 @@
         <v>—</v>
       </c>
       <c r="K30" t="str">
-        <v>$0.0308/张</v>
+        <v>$0.0339/张</v>
       </c>
       <c r="L30" t="str">
         <v>✅</v>
       </c>
       <c r="M30" t="str">
-        <v>⚠-9%</v>
+        <v>✅</v>
       </c>
       <c r="N30" t="str">
         <v>—</v>
@@ -1990,33 +1990,33 @@
         <v>价✅</v>
       </c>
       <c r="Q30" t="str">
-        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>kling-2.1</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v>kling-2.1</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>可灵</v>
       </c>
       <c r="D31" t="str">
-        <v/>
+        <v>可灵</v>
       </c>
       <c r="E31" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F31" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="G31" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="H31" t="str">
-        <v>$0.056/张</v>
+        <v>$0.014/张</v>
       </c>
       <c r="I31" t="str">
         <v>—</v>
@@ -2025,7 +2025,7 @@
         <v>—</v>
       </c>
       <c r="K31" t="str">
-        <v>$0.055172/张</v>
+        <v>$0.013793/张</v>
       </c>
       <c r="L31" t="str">
         <v>✅</v>
@@ -2048,28 +2048,28 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>kling-3.0-omni</v>
+        <v/>
       </c>
       <c r="B32" t="str">
-        <v>kling-3.0-omni</v>
+        <v/>
       </c>
       <c r="C32" t="str">
-        <v>可灵</v>
+        <v/>
       </c>
       <c r="D32" t="str">
-        <v>可灵</v>
+        <v/>
       </c>
       <c r="E32" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F32" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="G32" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.1/张</v>
       </c>
       <c r="H32" t="str">
-        <v>$0.028/张</v>
+        <v>$0.014/张</v>
       </c>
       <c r="I32" t="str">
         <v>—</v>
@@ -2078,7 +2078,7 @@
         <v>—</v>
       </c>
       <c r="K32" t="str">
-        <v>$0.0308/张</v>
+        <v>$0.077241/张</v>
       </c>
       <c r="L32" t="str">
         <v>✅</v>
@@ -2093,7 +2093,7 @@
         <v>—</v>
       </c>
       <c r="P32" t="str">
-        <v>价✅</v>
+        <v>🔍待核验 价⚠+402.1%</v>
       </c>
       <c r="Q32" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
@@ -2113,16 +2113,16 @@
         <v/>
       </c>
       <c r="E33" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F33" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.26/张</v>
       </c>
       <c r="G33" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.26/张</v>
       </c>
       <c r="H33" t="str">
-        <v>$0.028/张</v>
+        <v>$0.037/张</v>
       </c>
       <c r="I33" t="str">
         <v>—</v>
@@ -2131,13 +2131,13 @@
         <v>—</v>
       </c>
       <c r="K33" t="str">
-        <v>$0.0308/张</v>
+        <v>—</v>
       </c>
       <c r="L33" t="str">
         <v>✅</v>
       </c>
       <c r="M33" t="str">
-        <v>⚠-9%</v>
+        <v>⚠-7.5%</v>
       </c>
       <c r="N33" t="str">
         <v>—</v>
@@ -2146,7 +2146,7 @@
         <v>—</v>
       </c>
       <c r="P33" t="str">
-        <v>价✅</v>
+        <v>ℹ 线上无同档刊例</v>
       </c>
       <c r="Q33" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
@@ -2154,28 +2154,28 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v/>
+        <v>kling-3</v>
       </c>
       <c r="B34" t="str">
-        <v/>
+        <v>kling-3.0</v>
       </c>
       <c r="C34" t="str">
-        <v/>
+        <v>可灵</v>
       </c>
       <c r="D34" t="str">
-        <v/>
+        <v>可灵</v>
       </c>
       <c r="E34" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F34" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="G34" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="H34" t="str">
-        <v>$0.056/张</v>
+        <v>$0.028/张</v>
       </c>
       <c r="I34" t="str">
         <v>—</v>
@@ -2184,7 +2184,7 @@
         <v>—</v>
       </c>
       <c r="K34" t="str">
-        <v>$0.055172/张</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="L34" t="str">
         <v>✅</v>
@@ -2199,7 +2199,7 @@
         <v>—</v>
       </c>
       <c r="P34" t="str">
-        <v>价⚠-10.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q34" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
@@ -2207,19 +2207,19 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>kling-o1</v>
+        <v/>
       </c>
       <c r="B35" t="str">
-        <v>kling-o1</v>
+        <v/>
       </c>
       <c r="C35" t="str">
-        <v>可灵</v>
+        <v/>
       </c>
       <c r="D35" t="str">
-        <v>可灵</v>
+        <v/>
       </c>
       <c r="E35" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F35" t="str">
         <v>¥0.2/张</v>
@@ -2272,16 +2272,16 @@
         <v/>
       </c>
       <c r="E36" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F36" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.4/张</v>
       </c>
       <c r="G36" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.4/张</v>
       </c>
       <c r="H36" t="str">
-        <v>$0.028/张</v>
+        <v>$0.056/张</v>
       </c>
       <c r="I36" t="str">
         <v>—</v>
@@ -2290,7 +2290,7 @@
         <v>—</v>
       </c>
       <c r="K36" t="str">
-        <v>$0.0308/张</v>
+        <v>$0.055172/张</v>
       </c>
       <c r="L36" t="str">
         <v>✅</v>
@@ -2305,7 +2305,7 @@
         <v>—</v>
       </c>
       <c r="P36" t="str">
-        <v>价✅</v>
+        <v>价⚠-10.3%</v>
       </c>
       <c r="Q36" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
@@ -2313,28 +2313,28 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v/>
+        <v>kling-3.0-omni</v>
       </c>
       <c r="B37" t="str">
-        <v/>
+        <v>kling-3.0-omni</v>
       </c>
       <c r="C37" t="str">
-        <v/>
+        <v>可灵</v>
       </c>
       <c r="D37" t="str">
-        <v/>
+        <v>可灵</v>
       </c>
       <c r="E37" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F37" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="G37" t="str">
-        <v>¥0.4/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="H37" t="str">
-        <v>$0.056/张</v>
+        <v>$0.028/张</v>
       </c>
       <c r="I37" t="str">
         <v>—</v>
@@ -2343,7 +2343,7 @@
         <v>—</v>
       </c>
       <c r="K37" t="str">
-        <v>$0.055172/张</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="L37" t="str">
         <v>✅</v>
@@ -2358,7 +2358,7 @@
         <v>—</v>
       </c>
       <c r="P37" t="str">
-        <v>价⚠-10.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q37" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
@@ -2366,28 +2366,28 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>hunyuan-image-3</v>
+        <v/>
       </c>
       <c r="B38" t="str">
-        <v>hunyuan-3.0</v>
+        <v/>
       </c>
       <c r="C38" t="str">
-        <v>混元</v>
+        <v/>
       </c>
       <c r="D38" t="str">
-        <v>混元</v>
+        <v/>
       </c>
       <c r="E38" t="str">
-        <v>输出</v>
+        <v>2K</v>
       </c>
       <c r="F38" t="str">
         <v>¥0.2/张</v>
       </c>
       <c r="G38" t="str">
-        <v>—</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="H38" t="str">
-        <v>—</v>
+        <v>$0.028/张</v>
       </c>
       <c r="I38" t="str">
         <v>—</v>
@@ -2396,13 +2396,13 @@
         <v>—</v>
       </c>
       <c r="K38" t="str">
-        <v>—</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="L38" t="str">
-        <v>—</v>
+        <v>✅</v>
       </c>
       <c r="M38" t="str">
-        <v>—</v>
+        <v>⚠-9%</v>
       </c>
       <c r="N38" t="str">
         <v>—</v>
@@ -2411,36 +2411,36 @@
         <v>—</v>
       </c>
       <c r="P38" t="str">
-        <v>ℹ 线上无同档刊例</v>
+        <v>价✅</v>
       </c>
       <c r="Q38" t="str">
-        <v>Trinity Hunyuan-3.0 · 官方与 hy-image-v3.0 同价 0.2元/张</v>
+        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>hy-image-lite</v>
+        <v/>
       </c>
       <c r="B39" t="str">
-        <v>hy-image-lite</v>
+        <v/>
       </c>
       <c r="C39" t="str">
-        <v>混元</v>
+        <v/>
       </c>
       <c r="D39" t="str">
-        <v>混元</v>
+        <v/>
       </c>
       <c r="E39" t="str">
-        <v>输出</v>
+        <v>4K</v>
       </c>
       <c r="F39" t="str">
-        <v>¥0.099/张</v>
+        <v>¥0.4/张</v>
       </c>
       <c r="G39" t="str">
-        <v>—</v>
+        <v>¥0.4/张</v>
       </c>
       <c r="H39" t="str">
-        <v>—</v>
+        <v>$0.056/张</v>
       </c>
       <c r="I39" t="str">
         <v>—</v>
@@ -2449,13 +2449,13 @@
         <v>—</v>
       </c>
       <c r="K39" t="str">
-        <v>—</v>
+        <v>$0.055172/张</v>
       </c>
       <c r="L39" t="str">
-        <v>—</v>
+        <v>✅</v>
       </c>
       <c r="M39" t="str">
-        <v>—</v>
+        <v>⚠-9%</v>
       </c>
       <c r="N39" t="str">
         <v>—</v>
@@ -2464,36 +2464,36 @@
         <v>—</v>
       </c>
       <c r="P39" t="str">
-        <v>— 未上架</v>
+        <v>价⚠-10.3%</v>
       </c>
       <c r="Q39" t="str">
-        <v>TokenHub hy-image-lite · 混元生图极速版</v>
+        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>hy-image-v3.0</v>
+        <v>kling-o1</v>
       </c>
       <c r="B40" t="str">
-        <v>hy-image-v3.0</v>
+        <v>kling-o1</v>
       </c>
       <c r="C40" t="str">
-        <v>混元</v>
+        <v>可灵</v>
       </c>
       <c r="D40" t="str">
-        <v>混元</v>
+        <v>可灵</v>
       </c>
       <c r="E40" t="str">
-        <v>输出</v>
+        <v>1K</v>
       </c>
       <c r="F40" t="str">
         <v>¥0.2/张</v>
       </c>
       <c r="G40" t="str">
-        <v>—</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="H40" t="str">
-        <v>—</v>
+        <v>$0.028/张</v>
       </c>
       <c r="I40" t="str">
         <v>—</v>
@@ -2502,13 +2502,13 @@
         <v>—</v>
       </c>
       <c r="K40" t="str">
-        <v>—</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="L40" t="str">
-        <v>—</v>
+        <v>✅</v>
       </c>
       <c r="M40" t="str">
-        <v>—</v>
+        <v>⚠-9%</v>
       </c>
       <c r="N40" t="str">
         <v>—</v>
@@ -2517,27 +2517,27 @@
         <v>—</v>
       </c>
       <c r="P40" t="str">
-        <v>— 未上架</v>
+        <v>价✅</v>
       </c>
       <c r="Q40" t="str">
-        <v>TokenHub hy-image-v3.0 · API 混元生图 3.0</v>
+        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>doubao-seedream-4.0</v>
+        <v/>
       </c>
       <c r="B41" t="str">
-        <v>si-4.0</v>
+        <v/>
       </c>
       <c r="C41" t="str">
-        <v>豆包</v>
+        <v/>
       </c>
       <c r="D41" t="str">
-        <v>豆包</v>
+        <v/>
       </c>
       <c r="E41" t="str">
-        <v>1K</v>
+        <v>2K</v>
       </c>
       <c r="F41" t="str">
         <v>¥0.2/张</v>
@@ -2546,13 +2546,13 @@
         <v>¥0.2/张</v>
       </c>
       <c r="H41" t="str">
-        <v>$0.0308/张</v>
+        <v>$0.028/张</v>
       </c>
       <c r="I41" t="str">
         <v>—</v>
       </c>
       <c r="J41" t="str">
-        <v>¥0.2/张</v>
+        <v>—</v>
       </c>
       <c r="K41" t="str">
         <v>$0.0308/张</v>
@@ -2561,19 +2561,19 @@
         <v>✅</v>
       </c>
       <c r="M41" t="str">
-        <v>✅</v>
+        <v>⚠-9%</v>
       </c>
       <c r="N41" t="str">
         <v>—</v>
       </c>
       <c r="O41" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P41" t="str">
         <v>价✅</v>
       </c>
       <c r="Q41" t="str">
-        <v/>
+        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
       </c>
     </row>
     <row r="42">
@@ -2590,149 +2590,149 @@
         <v/>
       </c>
       <c r="E42" t="str">
-        <v>2K</v>
+        <v>4K</v>
       </c>
       <c r="F42" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.4/张</v>
       </c>
       <c r="G42" t="str">
-        <v>¥0.2/张</v>
+        <v>¥0.4/张</v>
       </c>
       <c r="H42" t="str">
-        <v>$0.0308/张</v>
+        <v>$0.056/张</v>
       </c>
       <c r="I42" t="str">
         <v>—</v>
       </c>
       <c r="J42" t="str">
-        <v>¥0.2/张</v>
+        <v>—</v>
       </c>
       <c r="K42" t="str">
-        <v>$0.0308/张</v>
+        <v>$0.055172/张</v>
       </c>
       <c r="L42" t="str">
         <v>✅</v>
       </c>
       <c r="M42" t="str">
-        <v>✅</v>
+        <v>⚠-9%</v>
       </c>
       <c r="N42" t="str">
         <v>—</v>
       </c>
       <c r="O42" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P42" t="str">
-        <v>价✅</v>
+        <v>价⚠-10.3%</v>
       </c>
       <c r="Q42" t="str">
-        <v/>
+        <v>灵感值/Credits 计价，无公开按张 API 价目</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v/>
+        <v>hunyuan-image-3</v>
       </c>
       <c r="B43" t="str">
-        <v/>
+        <v>hunyuan-3.0</v>
       </c>
       <c r="C43" t="str">
-        <v/>
+        <v>混元</v>
       </c>
       <c r="D43" t="str">
-        <v/>
+        <v>混元</v>
       </c>
       <c r="E43" t="str">
-        <v>4K</v>
+        <v>输出</v>
       </c>
       <c r="F43" t="str">
         <v>¥0.2/张</v>
       </c>
       <c r="G43" t="str">
-        <v>¥0.2/张</v>
+        <v>—</v>
       </c>
       <c r="H43" t="str">
-        <v>$0.0308/张</v>
+        <v>—</v>
       </c>
       <c r="I43" t="str">
         <v>—</v>
       </c>
       <c r="J43" t="str">
-        <v>¥0.2/张</v>
+        <v>—</v>
       </c>
       <c r="K43" t="str">
-        <v>$0.0308/张</v>
+        <v>—</v>
       </c>
       <c r="L43" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M43" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N43" t="str">
         <v>—</v>
       </c>
       <c r="O43" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P43" t="str">
-        <v>价✅</v>
+        <v>ℹ 线上无同档刊例</v>
       </c>
       <c r="Q43" t="str">
-        <v/>
+        <v>Trinity Hunyuan-3.0 · 官方与 hy-image-v3.0 同价 0.2元/张</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>doubao-seedream-4.5</v>
+        <v/>
       </c>
       <c r="B44" t="str">
-        <v>si-4.5</v>
+        <v/>
       </c>
       <c r="C44" t="str">
-        <v>豆包</v>
+        <v/>
       </c>
       <c r="D44" t="str">
-        <v>豆包</v>
+        <v/>
       </c>
       <c r="E44" t="str">
         <v>1K</v>
       </c>
       <c r="F44" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="G44" t="str">
-        <v>¥0.25/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="H44" t="str">
-        <v>$0.0385/张</v>
+        <v>—</v>
       </c>
       <c r="I44" t="str">
         <v>—</v>
       </c>
       <c r="J44" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="K44" t="str">
-        <v>$0.0385/张</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="L44" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M44" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N44" t="str">
         <v>—</v>
       </c>
       <c r="O44" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P44" t="str">
-        <v>价✅</v>
+        <v>—</v>
       </c>
       <c r="Q44" t="str">
-        <v/>
+        <v>Trinity Hunyuan-3.0 · 官方与 hy-image-v3.0 同价 0.2元/张</v>
       </c>
     </row>
     <row r="45">
@@ -2752,40 +2752,40 @@
         <v>2K</v>
       </c>
       <c r="F45" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="G45" t="str">
-        <v>¥0.25/张</v>
+        <v>¥0.28/张</v>
       </c>
       <c r="H45" t="str">
-        <v>$0.0385/张</v>
+        <v>—</v>
       </c>
       <c r="I45" t="str">
         <v>—</v>
       </c>
       <c r="J45" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="K45" t="str">
-        <v>$0.0385/张</v>
+        <v>$0.0431/张</v>
       </c>
       <c r="L45" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M45" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N45" t="str">
         <v>—</v>
       </c>
       <c r="O45" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P45" t="str">
-        <v>价✅</v>
+        <v>—</v>
       </c>
       <c r="Q45" t="str">
-        <v/>
+        <v>Trinity Hunyuan-3.0 · 官方与 hy-image-v3.0 同价 0.2元/张</v>
       </c>
     </row>
     <row r="46">
@@ -2805,181 +2805,181 @@
         <v>4K</v>
       </c>
       <c r="F46" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="G46" t="str">
-        <v>¥0.25/张</v>
+        <v>¥0.36/张</v>
       </c>
       <c r="H46" t="str">
-        <v>$0.0385/张</v>
+        <v>—</v>
       </c>
       <c r="I46" t="str">
         <v>—</v>
       </c>
       <c r="J46" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="K46" t="str">
-        <v>$0.0385/张</v>
+        <v>$0.049655/张</v>
       </c>
       <c r="L46" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M46" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N46" t="str">
         <v>—</v>
       </c>
       <c r="O46" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P46" t="str">
-        <v>价✅</v>
+        <v>—</v>
       </c>
       <c r="Q46" t="str">
-        <v/>
+        <v>Trinity Hunyuan-3.0 · 官方与 hy-image-v3.0 同价 0.2元/张</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>doubao-seedream-5.0-lite</v>
+        <v>hy-image-lite</v>
       </c>
       <c r="B47" t="str">
-        <v>si-5.0-lite</v>
+        <v>hy-image-lite</v>
       </c>
       <c r="C47" t="str">
-        <v>豆包</v>
+        <v>混元</v>
       </c>
       <c r="D47" t="str">
-        <v>豆包</v>
+        <v>混元</v>
       </c>
       <c r="E47" t="str">
-        <v>1K</v>
+        <v>输出</v>
       </c>
       <c r="F47" t="str">
-        <v>¥0.22/张</v>
+        <v>¥0.099/张</v>
       </c>
       <c r="G47" t="str">
-        <v>¥0.22/张</v>
+        <v>—</v>
       </c>
       <c r="H47" t="str">
-        <v>$0.0339/张</v>
+        <v>—</v>
       </c>
       <c r="I47" t="str">
         <v>—</v>
       </c>
       <c r="J47" t="str">
-        <v>¥0.22/张</v>
+        <v>—</v>
       </c>
       <c r="K47" t="str">
-        <v>$0.0339/张</v>
+        <v>—</v>
       </c>
       <c r="L47" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M47" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N47" t="str">
         <v>—</v>
       </c>
       <c r="O47" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P47" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q47" t="str">
-        <v/>
+        <v>TokenHub hy-image-lite · 混元生图极速版</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v/>
+        <v>hy-image-v3.0</v>
       </c>
       <c r="B48" t="str">
-        <v/>
+        <v>hy-image-v3.0</v>
       </c>
       <c r="C48" t="str">
-        <v/>
+        <v>混元</v>
       </c>
       <c r="D48" t="str">
-        <v/>
+        <v>混元</v>
       </c>
       <c r="E48" t="str">
-        <v>2K</v>
+        <v>输出</v>
       </c>
       <c r="F48" t="str">
-        <v>¥0.22/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="G48" t="str">
-        <v>¥0.22/张</v>
+        <v>—</v>
       </c>
       <c r="H48" t="str">
-        <v>$0.0339/张</v>
+        <v>—</v>
       </c>
       <c r="I48" t="str">
         <v>—</v>
       </c>
       <c r="J48" t="str">
-        <v>¥0.22/张</v>
+        <v>—</v>
       </c>
       <c r="K48" t="str">
-        <v>$0.0339/张</v>
+        <v>—</v>
       </c>
       <c r="L48" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="M48" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="N48" t="str">
         <v>—</v>
       </c>
       <c r="O48" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P48" t="str">
-        <v>价✅</v>
+        <v>— 未上架</v>
       </c>
       <c r="Q48" t="str">
-        <v/>
+        <v>TokenHub hy-image-v3.0 · API 混元生图 3.0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v/>
+        <v>doubao-seedream-4.0</v>
       </c>
       <c r="B49" t="str">
-        <v/>
+        <v>si-4.0</v>
       </c>
       <c r="C49" t="str">
-        <v/>
+        <v>豆包</v>
       </c>
       <c r="D49" t="str">
-        <v/>
+        <v>豆包</v>
       </c>
       <c r="E49" t="str">
-        <v>4K</v>
+        <v>1K</v>
       </c>
       <c r="F49" t="str">
-        <v>¥0.22/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="G49" t="str">
-        <v>¥0.22/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="H49" t="str">
-        <v>$0.0339/张</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="I49" t="str">
         <v>—</v>
       </c>
       <c r="J49" t="str">
-        <v>¥0.22/张</v>
+        <v>¥0.2/张</v>
       </c>
       <c r="K49" t="str">
-        <v>$0.0339/张</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="L49" t="str">
         <v>✅</v>
@@ -3002,60 +3002,643 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
+        <v/>
+      </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v>2K</v>
+      </c>
+      <c r="F50" t="str">
+        <v>¥0.2/张</v>
+      </c>
+      <c r="G50" t="str">
+        <v>¥0.2/张</v>
+      </c>
+      <c r="H50" t="str">
+        <v>$0.0308/张</v>
+      </c>
+      <c r="I50" t="str">
+        <v>—</v>
+      </c>
+      <c r="J50" t="str">
+        <v>¥0.2/张</v>
+      </c>
+      <c r="K50" t="str">
+        <v>$0.0308/张</v>
+      </c>
+      <c r="L50" t="str">
+        <v>✅</v>
+      </c>
+      <c r="M50" t="str">
+        <v>✅</v>
+      </c>
+      <c r="N50" t="str">
+        <v>—</v>
+      </c>
+      <c r="O50" t="str">
+        <v>✅</v>
+      </c>
+      <c r="P50" t="str">
+        <v>价✅</v>
+      </c>
+      <c r="Q50" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v/>
+      </c>
+      <c r="B51" t="str">
+        <v/>
+      </c>
+      <c r="C51" t="str">
+        <v/>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51" t="str">
+        <v>4K</v>
+      </c>
+      <c r="F51" t="str">
+        <v>¥0.2/张</v>
+      </c>
+      <c r="G51" t="str">
+        <v>¥0.2/张</v>
+      </c>
+      <c r="H51" t="str">
+        <v>$0.0308/张</v>
+      </c>
+      <c r="I51" t="str">
+        <v>—</v>
+      </c>
+      <c r="J51" t="str">
+        <v>¥0.2/张</v>
+      </c>
+      <c r="K51" t="str">
+        <v>$0.0308/张</v>
+      </c>
+      <c r="L51" t="str">
+        <v>✅</v>
+      </c>
+      <c r="M51" t="str">
+        <v>✅</v>
+      </c>
+      <c r="N51" t="str">
+        <v>—</v>
+      </c>
+      <c r="O51" t="str">
+        <v>✅</v>
+      </c>
+      <c r="P51" t="str">
+        <v>价✅</v>
+      </c>
+      <c r="Q51" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>doubao-seedream-4.5</v>
+      </c>
+      <c r="B52" t="str">
+        <v>si-4.5</v>
+      </c>
+      <c r="C52" t="str">
+        <v>豆包</v>
+      </c>
+      <c r="D52" t="str">
+        <v>豆包</v>
+      </c>
+      <c r="E52" t="str">
+        <v>1K</v>
+      </c>
+      <c r="F52" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="G52" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="H52" t="str">
+        <v>$0.0385/张</v>
+      </c>
+      <c r="I52" t="str">
+        <v>—</v>
+      </c>
+      <c r="J52" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="K52" t="str">
+        <v>$0.0385/张</v>
+      </c>
+      <c r="L52" t="str">
+        <v>✅</v>
+      </c>
+      <c r="M52" t="str">
+        <v>✅</v>
+      </c>
+      <c r="N52" t="str">
+        <v>—</v>
+      </c>
+      <c r="O52" t="str">
+        <v>✅</v>
+      </c>
+      <c r="P52" t="str">
+        <v>价✅</v>
+      </c>
+      <c r="Q52" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v/>
+      </c>
+      <c r="B53" t="str">
+        <v/>
+      </c>
+      <c r="C53" t="str">
+        <v/>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v>2K</v>
+      </c>
+      <c r="F53" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="G53" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="H53" t="str">
+        <v>$0.0385/张</v>
+      </c>
+      <c r="I53" t="str">
+        <v>—</v>
+      </c>
+      <c r="J53" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="K53" t="str">
+        <v>$0.0385/张</v>
+      </c>
+      <c r="L53" t="str">
+        <v>✅</v>
+      </c>
+      <c r="M53" t="str">
+        <v>✅</v>
+      </c>
+      <c r="N53" t="str">
+        <v>—</v>
+      </c>
+      <c r="O53" t="str">
+        <v>✅</v>
+      </c>
+      <c r="P53" t="str">
+        <v>价✅</v>
+      </c>
+      <c r="Q53" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v/>
+      </c>
+      <c r="B54" t="str">
+        <v/>
+      </c>
+      <c r="C54" t="str">
+        <v/>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v>4K</v>
+      </c>
+      <c r="F54" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="G54" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="H54" t="str">
+        <v>$0.0385/张</v>
+      </c>
+      <c r="I54" t="str">
+        <v>—</v>
+      </c>
+      <c r="J54" t="str">
+        <v>¥0.25/张</v>
+      </c>
+      <c r="K54" t="str">
+        <v>$0.0385/张</v>
+      </c>
+      <c r="L54" t="str">
+        <v>✅</v>
+      </c>
+      <c r="M54" t="str">
+        <v>✅</v>
+      </c>
+      <c r="N54" t="str">
+        <v>—</v>
+      </c>
+      <c r="O54" t="str">
+        <v>✅</v>
+      </c>
+      <c r="P54" t="str">
+        <v>价✅</v>
+      </c>
+      <c r="Q54" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>doubao-seedream-5.0-lite</v>
+      </c>
+      <c r="B55" t="str">
+        <v>si-5.0-lite</v>
+      </c>
+      <c r="C55" t="str">
+        <v>豆包</v>
+      </c>
+      <c r="D55" t="str">
+        <v>豆包</v>
+      </c>
+      <c r="E55" t="str">
+        <v>1K</v>
+      </c>
+      <c r="F55" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="G55" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="H55" t="str">
+        <v>$0.0339/张</v>
+      </c>
+      <c r="I55" t="str">
+        <v>—</v>
+      </c>
+      <c r="J55" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="K55" t="str">
+        <v>$0.0339/张</v>
+      </c>
+      <c r="L55" t="str">
+        <v>✅</v>
+      </c>
+      <c r="M55" t="str">
+        <v>✅</v>
+      </c>
+      <c r="N55" t="str">
+        <v>—</v>
+      </c>
+      <c r="O55" t="str">
+        <v>✅</v>
+      </c>
+      <c r="P55" t="str">
+        <v>价✅</v>
+      </c>
+      <c r="Q55" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v/>
+      </c>
+      <c r="B56" t="str">
+        <v/>
+      </c>
+      <c r="C56" t="str">
+        <v/>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v>2K</v>
+      </c>
+      <c r="F56" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="G56" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="H56" t="str">
+        <v>$0.0339/张</v>
+      </c>
+      <c r="I56" t="str">
+        <v>—</v>
+      </c>
+      <c r="J56" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="K56" t="str">
+        <v>$0.0339/张</v>
+      </c>
+      <c r="L56" t="str">
+        <v>✅</v>
+      </c>
+      <c r="M56" t="str">
+        <v>✅</v>
+      </c>
+      <c r="N56" t="str">
+        <v>—</v>
+      </c>
+      <c r="O56" t="str">
+        <v>✅</v>
+      </c>
+      <c r="P56" t="str">
+        <v>价✅</v>
+      </c>
+      <c r="Q56" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v/>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v>4K</v>
+      </c>
+      <c r="F57" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="G57" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="H57" t="str">
+        <v>$0.0339/张</v>
+      </c>
+      <c r="I57" t="str">
+        <v>—</v>
+      </c>
+      <c r="J57" t="str">
+        <v>¥0.22/张</v>
+      </c>
+      <c r="K57" t="str">
+        <v>$0.0339/张</v>
+      </c>
+      <c r="L57" t="str">
+        <v>✅</v>
+      </c>
+      <c r="M57" t="str">
+        <v>✅</v>
+      </c>
+      <c r="N57" t="str">
+        <v>—</v>
+      </c>
+      <c r="O57" t="str">
+        <v>✅</v>
+      </c>
+      <c r="P57" t="str">
+        <v>价✅</v>
+      </c>
+      <c r="Q57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
         <v>qwen-image-0925</v>
       </c>
-      <c r="B50" t="str">
+      <c r="B58" t="str">
         <v>qwen-0925</v>
       </c>
-      <c r="C50" t="str">
+      <c r="C58" t="str">
         <v>通义</v>
       </c>
-      <c r="D50" t="str">
+      <c r="D58" t="str">
         <v>通义</v>
       </c>
-      <c r="E50" t="str">
+      <c r="E58" t="str">
         <v>输出</v>
       </c>
-      <c r="F50" t="str">
+      <c r="F58" t="str">
         <v>¥0.25/张</v>
       </c>
-      <c r="G50" t="str">
-        <v>—</v>
-      </c>
-      <c r="H50" t="str">
-        <v>—</v>
-      </c>
-      <c r="I50" t="str">
-        <v>—</v>
-      </c>
-      <c r="J50" t="str">
-        <v>—</v>
-      </c>
-      <c r="K50" t="str">
-        <v>—</v>
-      </c>
-      <c r="L50" t="str">
-        <v>—</v>
-      </c>
-      <c r="M50" t="str">
-        <v>—</v>
-      </c>
-      <c r="N50" t="str">
-        <v>—</v>
-      </c>
-      <c r="O50" t="str">
-        <v>—</v>
-      </c>
-      <c r="P50" t="str">
+      <c r="G58" t="str">
+        <v>—</v>
+      </c>
+      <c r="H58" t="str">
+        <v>—</v>
+      </c>
+      <c r="I58" t="str">
+        <v>—</v>
+      </c>
+      <c r="J58" t="str">
+        <v>—</v>
+      </c>
+      <c r="K58" t="str">
+        <v>—</v>
+      </c>
+      <c r="L58" t="str">
+        <v>—</v>
+      </c>
+      <c r="M58" t="str">
+        <v>—</v>
+      </c>
+      <c r="N58" t="str">
+        <v>—</v>
+      </c>
+      <c r="O58" t="str">
+        <v>—</v>
+      </c>
+      <c r="P58" t="str">
         <v>ℹ 线上无同档刊例</v>
       </c>
-      <c r="Q50" t="str">
+      <c r="Q58" t="str">
+        <v>Trinity qwen-0925 · 百炼 API qwen-image（统一 ¥0.25/张）</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v/>
+      </c>
+      <c r="B59" t="str">
+        <v/>
+      </c>
+      <c r="C59" t="str">
+        <v/>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59" t="str">
+        <v>1K</v>
+      </c>
+      <c r="F59" t="str">
+        <v>—</v>
+      </c>
+      <c r="G59" t="str">
+        <v>¥0.3/张</v>
+      </c>
+      <c r="H59" t="str">
+        <v>$0.0461538461538462/张</v>
+      </c>
+      <c r="I59" t="str">
+        <v>—</v>
+      </c>
+      <c r="J59" t="str">
+        <v>—</v>
+      </c>
+      <c r="K59" t="str">
+        <v>$0.0462/张</v>
+      </c>
+      <c r="L59" t="str">
+        <v>—</v>
+      </c>
+      <c r="M59" t="str">
+        <v>—</v>
+      </c>
+      <c r="N59" t="str">
+        <v>—</v>
+      </c>
+      <c r="O59" t="str">
+        <v>—</v>
+      </c>
+      <c r="P59" t="str">
+        <v>ℹ 官方无档 · 价✅</v>
+      </c>
+      <c r="Q59" t="str">
+        <v>Trinity qwen-0925 · 百炼 API qwen-image（统一 ¥0.25/张）</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v/>
+      </c>
+      <c r="B60" t="str">
+        <v/>
+      </c>
+      <c r="C60" t="str">
+        <v/>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60" t="str">
+        <v>2K</v>
+      </c>
+      <c r="F60" t="str">
+        <v>—</v>
+      </c>
+      <c r="G60" t="str">
+        <v>¥0.38/张</v>
+      </c>
+      <c r="H60" t="str">
+        <v>$0.0584615384615385/张</v>
+      </c>
+      <c r="I60" t="str">
+        <v>—</v>
+      </c>
+      <c r="J60" t="str">
+        <v>—</v>
+      </c>
+      <c r="K60" t="str">
+        <v>$0.052414/张</v>
+      </c>
+      <c r="L60" t="str">
+        <v>—</v>
+      </c>
+      <c r="M60" t="str">
+        <v>—</v>
+      </c>
+      <c r="N60" t="str">
+        <v>—</v>
+      </c>
+      <c r="O60" t="str">
+        <v>—</v>
+      </c>
+      <c r="P60" t="str">
+        <v>ℹ 官方无档 · 价⚠-10.3%</v>
+      </c>
+      <c r="Q60" t="str">
+        <v>Trinity qwen-0925 · 百炼 API qwen-image（统一 ¥0.25/张）</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v/>
+      </c>
+      <c r="B61" t="str">
+        <v/>
+      </c>
+      <c r="C61" t="str">
+        <v/>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v>4K</v>
+      </c>
+      <c r="F61" t="str">
+        <v>—</v>
+      </c>
+      <c r="G61" t="str">
+        <v>¥0.46/张</v>
+      </c>
+      <c r="H61" t="str">
+        <v>$0.0707692307692308/张</v>
+      </c>
+      <c r="I61" t="str">
+        <v>—</v>
+      </c>
+      <c r="J61" t="str">
+        <v>—</v>
+      </c>
+      <c r="K61" t="str">
+        <v>$0.063448/张</v>
+      </c>
+      <c r="L61" t="str">
+        <v>—</v>
+      </c>
+      <c r="M61" t="str">
+        <v>—</v>
+      </c>
+      <c r="N61" t="str">
+        <v>—</v>
+      </c>
+      <c r="O61" t="str">
+        <v>—</v>
+      </c>
+      <c r="P61" t="str">
+        <v>ℹ 官方无档 · 价⚠-10.3%</v>
+      </c>
+      <c r="Q61" t="str">
         <v>Trinity qwen-0925 · 百炼 API qwen-image（统一 ¥0.25/张）</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q61"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3461,7 +4044,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>生成时间：2026-07-03T10:15:33Z</v>
+        <v>生成时间：2026-07-06T10:45:38Z</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
feat(pricing): unify L4 compare exports and drop pipeline discount columns
Align text/image/video compare hub channels and sheet headers; remove
supplier-discounts.json and discount/cost columns from supplier tables
(margin and discounts belong in admin). Add supplier-cost-discounts
business ledger, modality online price caches, and rename the product
manual sidebar to 模型价目与刊例治理.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/pricing/output/trinity-pricing-image.xlsx
+++ b/pricing/output/trinity-pricing-image.xlsx
@@ -420,7 +420,7 @@
         <v>分辨率档</v>
       </c>
       <c r="F1" t="str">
-        <v>厂商官方</v>
+        <v>厂商官方价</v>
       </c>
       <c r="G1" t="str">
         <v>AIGC国内</v>
@@ -432,7 +432,7 @@
         <v>TokenHub</v>
       </c>
       <c r="J1" t="str">
-        <v>火山方舟</v>
+        <v>OpenRouter</v>
       </c>
       <c r="K1" t="str">
         <v>线上刊例</v>
@@ -447,7 +447,7 @@
         <v>TokenHub vs官方</v>
       </c>
       <c r="O1" t="str">
-        <v>火山vs官方</v>
+        <v>OpenRouter vs官方</v>
       </c>
       <c r="P1" t="str">
         <v>刊例结论</v>
@@ -488,7 +488,7 @@
         <v>—</v>
       </c>
       <c r="K2" t="str">
-        <v>$0.0414/张</v>
+        <v>$0.039/张</v>
       </c>
       <c r="L2" t="str">
         <v>—</v>
@@ -503,25 +503,13 @@
         <v>—</v>
       </c>
       <c r="P2" t="str">
-        <v>价⚠+6.2%</v>
+        <v>价✅</v>
       </c>
       <c r="Q2" t="str">
         <v>API ID gemini-2.5-flash-image · Nano Banana</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v/>
-      </c>
-      <c r="B3" t="str">
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
       <c r="E3" t="str">
         <v>2K</v>
       </c>
@@ -541,7 +529,7 @@
         <v>—</v>
       </c>
       <c r="K3" t="str">
-        <v>$0.0586/张</v>
+        <v>$0.051/张</v>
       </c>
       <c r="L3" t="str">
         <v>—</v>
@@ -556,25 +544,13 @@
         <v>—</v>
       </c>
       <c r="P3" t="str">
-        <v>ℹ 官方无档 · 价⚠+14.9%</v>
+        <v>ℹ 官方无档 · 价✅</v>
       </c>
       <c r="Q3" t="str">
         <v>API ID gemini-2.5-flash-image · Nano Banana</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v/>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
       <c r="E4" t="str">
         <v>4K</v>
       </c>
@@ -594,7 +570,7 @@
         <v>—</v>
       </c>
       <c r="K4" t="str">
-        <v>$0.0635/张</v>
+        <v>$0.063/张</v>
       </c>
       <c r="L4" t="str">
         <v>—</v>
@@ -609,7 +585,7 @@
         <v>—</v>
       </c>
       <c r="P4" t="str">
-        <v>ℹ 官方无档 · 价⚠+0.8%</v>
+        <v>ℹ 官方无档 · 价✅</v>
       </c>
       <c r="Q4" t="str">
         <v>API ID gemini-2.5-flash-image · Nano Banana</v>
@@ -647,7 +623,7 @@
         <v>—</v>
       </c>
       <c r="K5" t="str">
-        <v>$0.137931/张</v>
+        <v>$0.134/张</v>
       </c>
       <c r="L5" t="str">
         <v>—</v>
@@ -662,25 +638,13 @@
         <v>—</v>
       </c>
       <c r="P5" t="str">
-        <v>价⚠+2.9%</v>
+        <v>价✅</v>
       </c>
       <c r="Q5" t="str">
         <v>API ID gemini-3-pro-image · Nano Banana Pro</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v/>
-      </c>
-      <c r="B6" t="str">
-        <v/>
-      </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
       <c r="E6" t="str">
         <v>2K</v>
       </c>
@@ -700,7 +664,7 @@
         <v>—</v>
       </c>
       <c r="K6" t="str">
-        <v>$0.248276/张</v>
+        <v>$0.134/张</v>
       </c>
       <c r="L6" t="str">
         <v>—</v>
@@ -715,25 +679,13 @@
         <v>—</v>
       </c>
       <c r="P6" t="str">
-        <v>🔍待核验 价⚠+85.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q6" t="str">
         <v>API ID gemini-3-pro-image · Nano Banana Pro</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-      <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
       <c r="E7" t="str">
         <v>4K</v>
       </c>
@@ -828,18 +780,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
-        <v/>
-      </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
       <c r="E9" t="str">
         <v>1K</v>
       </c>
@@ -859,7 +799,7 @@
         <v>—</v>
       </c>
       <c r="K9" t="str">
-        <v>$0.077/张</v>
+        <v>$0.067/张</v>
       </c>
       <c r="L9" t="str">
         <v>—</v>
@@ -874,25 +814,13 @@
         <v>—</v>
       </c>
       <c r="P9" t="str">
-        <v>价⚠+14.9%</v>
+        <v>价✅</v>
       </c>
       <c r="Q9" t="str">
         <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
-        <v/>
-      </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
       <c r="E10" t="str">
         <v>2K</v>
       </c>
@@ -912,7 +840,7 @@
         <v>—</v>
       </c>
       <c r="K10" t="str">
-        <v>$0.1154/张</v>
+        <v>$0.101/张</v>
       </c>
       <c r="L10" t="str">
         <v>—</v>
@@ -927,25 +855,13 @@
         <v>—</v>
       </c>
       <c r="P10" t="str">
-        <v>价⚠+14.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q10" t="str">
         <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-      <c r="B11" t="str">
-        <v/>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
       <c r="E11" t="str">
         <v>4K</v>
       </c>
@@ -965,7 +881,7 @@
         <v>—</v>
       </c>
       <c r="K11" t="str">
-        <v>$0.154483/张</v>
+        <v>$0.151/张</v>
       </c>
       <c r="L11" t="str">
         <v>—</v>
@@ -980,25 +896,13 @@
         <v>—</v>
       </c>
       <c r="P11" t="str">
-        <v>价⚠+2.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q11" t="str">
         <v>API ID gemini-3.1-flash-image · Nano Banana 2</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <v/>
-      </c>
-      <c r="C12" t="str">
-        <v/>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
       <c r="E12" t="str">
         <v>1K以下</v>
       </c>
@@ -1071,7 +975,7 @@
         <v>—</v>
       </c>
       <c r="K13" t="str">
-        <v>$0.0462/张</v>
+        <v>$0.039/张</v>
       </c>
       <c r="L13" t="str">
         <v>—</v>
@@ -1086,25 +990,13 @@
         <v>—</v>
       </c>
       <c r="P13" t="str">
-        <v>价⚠+18.5%</v>
+        <v>价✅</v>
       </c>
       <c r="Q13" t="str">
         <v>订阅制，无公开 API 按张价目</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-      <c r="B14" t="str">
-        <v/>
-      </c>
-      <c r="C14" t="str">
-        <v/>
-      </c>
-      <c r="D14" t="str">
-        <v/>
-      </c>
       <c r="E14" t="str">
         <v>2K</v>
       </c>
@@ -1124,7 +1016,7 @@
         <v>—</v>
       </c>
       <c r="K14" t="str">
-        <v>$0.052414/张</v>
+        <v>$0.051/张</v>
       </c>
       <c r="L14" t="str">
         <v>—</v>
@@ -1139,25 +1031,13 @@
         <v>—</v>
       </c>
       <c r="P14" t="str">
-        <v>ℹ 官方无档 · 价⚠+2.8%</v>
+        <v>ℹ 官方无档 · 价✅</v>
       </c>
       <c r="Q14" t="str">
         <v>订阅制，无公开 API 按张价目</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="str">
-        <v/>
-      </c>
-      <c r="B15" t="str">
-        <v/>
-      </c>
-      <c r="C15" t="str">
-        <v/>
-      </c>
-      <c r="D15" t="str">
-        <v/>
-      </c>
       <c r="E15" t="str">
         <v>4K</v>
       </c>
@@ -1177,7 +1057,7 @@
         <v>—</v>
       </c>
       <c r="K15" t="str">
-        <v>$0.063448/张</v>
+        <v>$0.063/张</v>
       </c>
       <c r="L15" t="str">
         <v>—</v>
@@ -1192,7 +1072,7 @@
         <v>—</v>
       </c>
       <c r="P15" t="str">
-        <v>ℹ 官方无档 · 价⚠+0.7%</v>
+        <v>ℹ 官方无档 · 价✅</v>
       </c>
       <c r="Q15" t="str">
         <v>订阅制，无公开 API 按张价目</v>
@@ -1230,7 +1110,7 @@
         <v>—</v>
       </c>
       <c r="K16" t="str">
-        <v>$1.583/张</v>
+        <v>$0.211/张</v>
       </c>
       <c r="L16" t="str">
         <v>—</v>
@@ -1245,25 +1125,13 @@
         <v>—</v>
       </c>
       <c r="P16" t="str">
-        <v>🔍待核验 价⚠+650.2%</v>
+        <v>价✅</v>
       </c>
       <c r="Q16" t="str">
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="str">
-        <v/>
-      </c>
-      <c r="B17" t="str">
-        <v/>
-      </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <v/>
-      </c>
       <c r="E17" t="str">
         <v>2K</v>
       </c>
@@ -1283,7 +1151,7 @@
         <v>—</v>
       </c>
       <c r="K17" t="str">
-        <v>$3.21/张</v>
+        <v>$0.428/张</v>
       </c>
       <c r="L17" t="str">
         <v>—</v>
@@ -1298,25 +1166,13 @@
         <v>—</v>
       </c>
       <c r="P17" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>价✅</v>
       </c>
       <c r="Q17" t="str">
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="str">
-        <v/>
-      </c>
-      <c r="B18" t="str">
-        <v/>
-      </c>
-      <c r="C18" t="str">
-        <v/>
-      </c>
-      <c r="D18" t="str">
-        <v/>
-      </c>
       <c r="E18" t="str">
         <v>4K</v>
       </c>
@@ -1336,7 +1192,7 @@
         <v>—</v>
       </c>
       <c r="K18" t="str">
-        <v>$5.34/张</v>
+        <v>$0.712/张</v>
       </c>
       <c r="L18" t="str">
         <v>—</v>
@@ -1351,7 +1207,7 @@
         <v>—</v>
       </c>
       <c r="P18" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>价✅</v>
       </c>
       <c r="Q18" t="str">
         <v/>
@@ -1389,7 +1245,7 @@
         <v>—</v>
       </c>
       <c r="K19" t="str">
-        <v>$0.045/张</v>
+        <v>$0.006/张</v>
       </c>
       <c r="L19" t="str">
         <v>—</v>
@@ -1404,25 +1260,13 @@
         <v>—</v>
       </c>
       <c r="P19" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>价✅</v>
       </c>
       <c r="Q19" t="str">
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="str">
-        <v/>
-      </c>
-      <c r="B20" t="str">
-        <v/>
-      </c>
-      <c r="C20" t="str">
-        <v/>
-      </c>
-      <c r="D20" t="str">
-        <v/>
-      </c>
       <c r="E20" t="str">
         <v>2K</v>
       </c>
@@ -1442,7 +1286,7 @@
         <v>—</v>
       </c>
       <c r="K20" t="str">
-        <v>$0.09/张</v>
+        <v>$0.012/张</v>
       </c>
       <c r="L20" t="str">
         <v>—</v>
@@ -1457,25 +1301,13 @@
         <v>—</v>
       </c>
       <c r="P20" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>价✅</v>
       </c>
       <c r="Q20" t="str">
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="str">
-        <v/>
-      </c>
-      <c r="B21" t="str">
-        <v/>
-      </c>
-      <c r="C21" t="str">
-        <v/>
-      </c>
-      <c r="D21" t="str">
-        <v/>
-      </c>
       <c r="E21" t="str">
         <v>4K</v>
       </c>
@@ -1495,7 +1327,7 @@
         <v>—</v>
       </c>
       <c r="K21" t="str">
-        <v>$0.15/张</v>
+        <v>$0.02/张</v>
       </c>
       <c r="L21" t="str">
         <v>—</v>
@@ -1510,7 +1342,7 @@
         <v>—</v>
       </c>
       <c r="P21" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>价✅</v>
       </c>
       <c r="Q21" t="str">
         <v/>
@@ -1548,7 +1380,7 @@
         <v>—</v>
       </c>
       <c r="K22" t="str">
-        <v>$0.398/张</v>
+        <v>$0.053/张</v>
       </c>
       <c r="L22" t="str">
         <v>—</v>
@@ -1563,25 +1395,13 @@
         <v>—</v>
       </c>
       <c r="P22" t="str">
-        <v>🔍待核验 价⚠+650.9%</v>
+        <v>价✅</v>
       </c>
       <c r="Q22" t="str">
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="str">
-        <v/>
-      </c>
-      <c r="B23" t="str">
-        <v/>
-      </c>
-      <c r="C23" t="str">
-        <v/>
-      </c>
-      <c r="D23" t="str">
-        <v/>
-      </c>
       <c r="E23" t="str">
         <v>2K</v>
       </c>
@@ -1601,7 +1421,7 @@
         <v>—</v>
       </c>
       <c r="K23" t="str">
-        <v>$0.803/张</v>
+        <v>$0.107/张</v>
       </c>
       <c r="L23" t="str">
         <v>—</v>
@@ -1616,25 +1436,13 @@
         <v>—</v>
       </c>
       <c r="P23" t="str">
-        <v>🔍待核验 价⚠+650.5%</v>
+        <v>价✅</v>
       </c>
       <c r="Q23" t="str">
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="str">
-        <v/>
-      </c>
-      <c r="B24" t="str">
-        <v/>
-      </c>
-      <c r="C24" t="str">
-        <v/>
-      </c>
-      <c r="D24" t="str">
-        <v/>
-      </c>
       <c r="E24" t="str">
         <v>4K</v>
       </c>
@@ -1654,7 +1462,7 @@
         <v>—</v>
       </c>
       <c r="K24" t="str">
-        <v>$1.335/张</v>
+        <v>$0.178/张</v>
       </c>
       <c r="L24" t="str">
         <v>—</v>
@@ -1669,7 +1477,7 @@
         <v>—</v>
       </c>
       <c r="P24" t="str">
-        <v>🔍待核验 价⚠+650%</v>
+        <v>价✅</v>
       </c>
       <c r="Q24" t="str">
         <v/>
@@ -1707,7 +1515,7 @@
         <v>—</v>
       </c>
       <c r="K25" t="str">
-        <v>$0.0577/张</v>
+        <v>$0.0289/张</v>
       </c>
       <c r="L25" t="str">
         <v>✅</v>
@@ -1722,25 +1530,13 @@
         <v>—</v>
       </c>
       <c r="P25" t="str">
-        <v>🔍待核验 价⚠+100%</v>
+        <v>价✅</v>
       </c>
       <c r="Q25" t="str">
         <v>viduq2 文生图 · 积分计价</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="str">
-        <v/>
-      </c>
-      <c r="B26" t="str">
-        <v/>
-      </c>
-      <c r="C26" t="str">
-        <v/>
-      </c>
-      <c r="D26" t="str">
-        <v/>
-      </c>
       <c r="E26" t="str">
         <v>2K</v>
       </c>
@@ -1760,7 +1556,7 @@
         <v>—</v>
       </c>
       <c r="K26" t="str">
-        <v>$0.077/张</v>
+        <v>$0.0385/张</v>
       </c>
       <c r="L26" t="str">
         <v>✅</v>
@@ -1775,25 +1571,13 @@
         <v>—</v>
       </c>
       <c r="P26" t="str">
-        <v>🔍待核验 价⚠+100.2%</v>
+        <v>价✅</v>
       </c>
       <c r="Q26" t="str">
         <v>viduq2 文生图 · 积分计价</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="str">
-        <v/>
-      </c>
-      <c r="B27" t="str">
-        <v/>
-      </c>
-      <c r="C27" t="str">
-        <v/>
-      </c>
-      <c r="D27" t="str">
-        <v/>
-      </c>
       <c r="E27" t="str">
         <v>4K</v>
       </c>
@@ -1813,7 +1597,7 @@
         <v>—</v>
       </c>
       <c r="K27" t="str">
-        <v>$0.0482/张</v>
+        <v>$0.0481/张</v>
       </c>
       <c r="L27" t="str">
         <v>✅</v>
@@ -1888,18 +1672,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="str">
-        <v/>
-      </c>
-      <c r="B29" t="str">
-        <v/>
-      </c>
-      <c r="C29" t="str">
-        <v/>
-      </c>
-      <c r="D29" t="str">
-        <v/>
-      </c>
       <c r="E29" t="str">
         <v>2K</v>
       </c>
@@ -1941,18 +1713,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="str">
-        <v/>
-      </c>
-      <c r="B30" t="str">
-        <v/>
-      </c>
-      <c r="C30" t="str">
-        <v/>
-      </c>
-      <c r="D30" t="str">
-        <v/>
-      </c>
       <c r="E30" t="str">
         <v>4K</v>
       </c>
@@ -2025,7 +1785,7 @@
         <v>—</v>
       </c>
       <c r="K31" t="str">
-        <v>$0.013793/张</v>
+        <v>$0.0154/张</v>
       </c>
       <c r="L31" t="str">
         <v>✅</v>
@@ -2040,25 +1800,13 @@
         <v>—</v>
       </c>
       <c r="P31" t="str">
-        <v>价⚠-10.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q31" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="str">
-        <v/>
-      </c>
-      <c r="B32" t="str">
-        <v/>
-      </c>
-      <c r="C32" t="str">
-        <v/>
-      </c>
-      <c r="D32" t="str">
-        <v/>
-      </c>
       <c r="E32" t="str">
         <v>2K</v>
       </c>
@@ -2078,7 +1826,7 @@
         <v>—</v>
       </c>
       <c r="K32" t="str">
-        <v>$0.077241/张</v>
+        <v>$0.0154/张</v>
       </c>
       <c r="L32" t="str">
         <v>✅</v>
@@ -2093,25 +1841,13 @@
         <v>—</v>
       </c>
       <c r="P32" t="str">
-        <v>🔍待核验 价⚠+402.1%</v>
+        <v>价✅</v>
       </c>
       <c r="Q32" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="str">
-        <v/>
-      </c>
-      <c r="B33" t="str">
-        <v/>
-      </c>
-      <c r="C33" t="str">
-        <v/>
-      </c>
-      <c r="D33" t="str">
-        <v/>
-      </c>
       <c r="E33" t="str">
         <v>4K</v>
       </c>
@@ -2206,18 +1942,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="str">
-        <v/>
-      </c>
-      <c r="B35" t="str">
-        <v/>
-      </c>
-      <c r="C35" t="str">
-        <v/>
-      </c>
-      <c r="D35" t="str">
-        <v/>
-      </c>
       <c r="E35" t="str">
         <v>2K</v>
       </c>
@@ -2259,18 +1983,6 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="str">
-        <v/>
-      </c>
-      <c r="B36" t="str">
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <v/>
-      </c>
-      <c r="D36" t="str">
-        <v/>
-      </c>
       <c r="E36" t="str">
         <v>4K</v>
       </c>
@@ -2290,7 +2002,7 @@
         <v>—</v>
       </c>
       <c r="K36" t="str">
-        <v>$0.055172/张</v>
+        <v>$0.0616/张</v>
       </c>
       <c r="L36" t="str">
         <v>✅</v>
@@ -2305,7 +2017,7 @@
         <v>—</v>
       </c>
       <c r="P36" t="str">
-        <v>价⚠-10.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q36" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
@@ -2365,18 +2077,6 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="str">
-        <v/>
-      </c>
-      <c r="B38" t="str">
-        <v/>
-      </c>
-      <c r="C38" t="str">
-        <v/>
-      </c>
-      <c r="D38" t="str">
-        <v/>
-      </c>
       <c r="E38" t="str">
         <v>2K</v>
       </c>
@@ -2418,18 +2118,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="str">
-        <v/>
-      </c>
-      <c r="B39" t="str">
-        <v/>
-      </c>
-      <c r="C39" t="str">
-        <v/>
-      </c>
-      <c r="D39" t="str">
-        <v/>
-      </c>
       <c r="E39" t="str">
         <v>4K</v>
       </c>
@@ -2449,7 +2137,7 @@
         <v>—</v>
       </c>
       <c r="K39" t="str">
-        <v>$0.055172/张</v>
+        <v>$0.0616/张</v>
       </c>
       <c r="L39" t="str">
         <v>✅</v>
@@ -2464,7 +2152,7 @@
         <v>—</v>
       </c>
       <c r="P39" t="str">
-        <v>价⚠-10.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q39" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
@@ -2524,18 +2212,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="str">
-        <v/>
-      </c>
-      <c r="B41" t="str">
-        <v/>
-      </c>
-      <c r="C41" t="str">
-        <v/>
-      </c>
-      <c r="D41" t="str">
-        <v/>
-      </c>
       <c r="E41" t="str">
         <v>2K</v>
       </c>
@@ -2577,18 +2253,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="str">
-        <v/>
-      </c>
-      <c r="B42" t="str">
-        <v/>
-      </c>
-      <c r="C42" t="str">
-        <v/>
-      </c>
-      <c r="D42" t="str">
-        <v/>
-      </c>
       <c r="E42" t="str">
         <v>4K</v>
       </c>
@@ -2608,7 +2272,7 @@
         <v>—</v>
       </c>
       <c r="K42" t="str">
-        <v>$0.055172/张</v>
+        <v>$0.0616/张</v>
       </c>
       <c r="L42" t="str">
         <v>✅</v>
@@ -2623,7 +2287,7 @@
         <v>—</v>
       </c>
       <c r="P42" t="str">
-        <v>价⚠-10.3%</v>
+        <v>价✅</v>
       </c>
       <c r="Q42" t="str">
         <v>灵感值/Credits 计价，无公开按张 API 价目</v>
@@ -2683,18 +2347,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="str">
-        <v/>
-      </c>
-      <c r="B44" t="str">
-        <v/>
-      </c>
-      <c r="C44" t="str">
-        <v/>
-      </c>
-      <c r="D44" t="str">
-        <v/>
-      </c>
       <c r="E44" t="str">
         <v>1K</v>
       </c>
@@ -2736,18 +2388,6 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="str">
-        <v/>
-      </c>
-      <c r="B45" t="str">
-        <v/>
-      </c>
-      <c r="C45" t="str">
-        <v/>
-      </c>
-      <c r="D45" t="str">
-        <v/>
-      </c>
       <c r="E45" t="str">
         <v>2K</v>
       </c>
@@ -2767,7 +2407,7 @@
         <v>—</v>
       </c>
       <c r="K45" t="str">
-        <v>$0.0431/张</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="L45" t="str">
         <v>—</v>
@@ -2789,18 +2429,6 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="str">
-        <v/>
-      </c>
-      <c r="B46" t="str">
-        <v/>
-      </c>
-      <c r="C46" t="str">
-        <v/>
-      </c>
-      <c r="D46" t="str">
-        <v/>
-      </c>
       <c r="E46" t="str">
         <v>4K</v>
       </c>
@@ -2820,7 +2448,7 @@
         <v>—</v>
       </c>
       <c r="K46" t="str">
-        <v>$0.049655/张</v>
+        <v>$0.0308/张</v>
       </c>
       <c r="L46" t="str">
         <v>—</v>
@@ -2976,7 +2604,7 @@
         <v>—</v>
       </c>
       <c r="J49" t="str">
-        <v>¥0.2/张</v>
+        <v>—</v>
       </c>
       <c r="K49" t="str">
         <v>$0.0308/张</v>
@@ -2991,7 +2619,7 @@
         <v>—</v>
       </c>
       <c r="O49" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P49" t="str">
         <v>价✅</v>
@@ -3001,18 +2629,6 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="str">
-        <v/>
-      </c>
-      <c r="B50" t="str">
-        <v/>
-      </c>
-      <c r="C50" t="str">
-        <v/>
-      </c>
-      <c r="D50" t="str">
-        <v/>
-      </c>
       <c r="E50" t="str">
         <v>2K</v>
       </c>
@@ -3029,7 +2645,7 @@
         <v>—</v>
       </c>
       <c r="J50" t="str">
-        <v>¥0.2/张</v>
+        <v>—</v>
       </c>
       <c r="K50" t="str">
         <v>$0.0308/张</v>
@@ -3044,7 +2660,7 @@
         <v>—</v>
       </c>
       <c r="O50" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P50" t="str">
         <v>价✅</v>
@@ -3054,18 +2670,6 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="str">
-        <v/>
-      </c>
-      <c r="B51" t="str">
-        <v/>
-      </c>
-      <c r="C51" t="str">
-        <v/>
-      </c>
-      <c r="D51" t="str">
-        <v/>
-      </c>
       <c r="E51" t="str">
         <v>4K</v>
       </c>
@@ -3082,7 +2686,7 @@
         <v>—</v>
       </c>
       <c r="J51" t="str">
-        <v>¥0.2/张</v>
+        <v>—</v>
       </c>
       <c r="K51" t="str">
         <v>$0.0308/张</v>
@@ -3097,7 +2701,7 @@
         <v>—</v>
       </c>
       <c r="O51" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P51" t="str">
         <v>价✅</v>
@@ -3135,7 +2739,7 @@
         <v>—</v>
       </c>
       <c r="J52" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="K52" t="str">
         <v>$0.0385/张</v>
@@ -3150,7 +2754,7 @@
         <v>—</v>
       </c>
       <c r="O52" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P52" t="str">
         <v>价✅</v>
@@ -3160,18 +2764,6 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="str">
-        <v/>
-      </c>
-      <c r="B53" t="str">
-        <v/>
-      </c>
-      <c r="C53" t="str">
-        <v/>
-      </c>
-      <c r="D53" t="str">
-        <v/>
-      </c>
       <c r="E53" t="str">
         <v>2K</v>
       </c>
@@ -3188,7 +2780,7 @@
         <v>—</v>
       </c>
       <c r="J53" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="K53" t="str">
         <v>$0.0385/张</v>
@@ -3203,7 +2795,7 @@
         <v>—</v>
       </c>
       <c r="O53" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P53" t="str">
         <v>价✅</v>
@@ -3213,18 +2805,6 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="str">
-        <v/>
-      </c>
-      <c r="B54" t="str">
-        <v/>
-      </c>
-      <c r="C54" t="str">
-        <v/>
-      </c>
-      <c r="D54" t="str">
-        <v/>
-      </c>
       <c r="E54" t="str">
         <v>4K</v>
       </c>
@@ -3241,7 +2821,7 @@
         <v>—</v>
       </c>
       <c r="J54" t="str">
-        <v>¥0.25/张</v>
+        <v>—</v>
       </c>
       <c r="K54" t="str">
         <v>$0.0385/张</v>
@@ -3256,7 +2836,7 @@
         <v>—</v>
       </c>
       <c r="O54" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P54" t="str">
         <v>价✅</v>
@@ -3294,7 +2874,7 @@
         <v>—</v>
       </c>
       <c r="J55" t="str">
-        <v>¥0.22/张</v>
+        <v>—</v>
       </c>
       <c r="K55" t="str">
         <v>$0.0339/张</v>
@@ -3309,7 +2889,7 @@
         <v>—</v>
       </c>
       <c r="O55" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P55" t="str">
         <v>价✅</v>
@@ -3319,18 +2899,6 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="str">
-        <v/>
-      </c>
-      <c r="B56" t="str">
-        <v/>
-      </c>
-      <c r="C56" t="str">
-        <v/>
-      </c>
-      <c r="D56" t="str">
-        <v/>
-      </c>
       <c r="E56" t="str">
         <v>2K</v>
       </c>
@@ -3347,7 +2915,7 @@
         <v>—</v>
       </c>
       <c r="J56" t="str">
-        <v>¥0.22/张</v>
+        <v>—</v>
       </c>
       <c r="K56" t="str">
         <v>$0.0339/张</v>
@@ -3362,7 +2930,7 @@
         <v>—</v>
       </c>
       <c r="O56" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P56" t="str">
         <v>价✅</v>
@@ -3372,18 +2940,6 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="str">
-        <v/>
-      </c>
-      <c r="B57" t="str">
-        <v/>
-      </c>
-      <c r="C57" t="str">
-        <v/>
-      </c>
-      <c r="D57" t="str">
-        <v/>
-      </c>
       <c r="E57" t="str">
         <v>4K</v>
       </c>
@@ -3400,7 +2956,7 @@
         <v>—</v>
       </c>
       <c r="J57" t="str">
-        <v>¥0.22/张</v>
+        <v>—</v>
       </c>
       <c r="K57" t="str">
         <v>$0.0339/张</v>
@@ -3415,7 +2971,7 @@
         <v>—</v>
       </c>
       <c r="O57" t="str">
-        <v>✅</v>
+        <v>—</v>
       </c>
       <c r="P57" t="str">
         <v>价✅</v>
@@ -3478,18 +3034,6 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="str">
-        <v/>
-      </c>
-      <c r="B59" t="str">
-        <v/>
-      </c>
-      <c r="C59" t="str">
-        <v/>
-      </c>
-      <c r="D59" t="str">
-        <v/>
-      </c>
       <c r="E59" t="str">
         <v>1K</v>
       </c>
@@ -3509,7 +3053,7 @@
         <v>—</v>
       </c>
       <c r="K59" t="str">
-        <v>$0.0462/张</v>
+        <v>$0.0385/张</v>
       </c>
       <c r="L59" t="str">
         <v>—</v>
@@ -3524,25 +3068,13 @@
         <v>—</v>
       </c>
       <c r="P59" t="str">
-        <v>ℹ 官方无档 · 价✅</v>
+        <v>ℹ 官方无档 · 价⚠-16.6%</v>
       </c>
       <c r="Q59" t="str">
         <v>Trinity qwen-0925 · 百炼 API qwen-image（统一 ¥0.25/张）</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="str">
-        <v/>
-      </c>
-      <c r="B60" t="str">
-        <v/>
-      </c>
-      <c r="C60" t="str">
-        <v/>
-      </c>
-      <c r="D60" t="str">
-        <v/>
-      </c>
       <c r="E60" t="str">
         <v>2K</v>
       </c>
@@ -3562,7 +3094,7 @@
         <v>—</v>
       </c>
       <c r="K60" t="str">
-        <v>$0.052414/张</v>
+        <v>$0.0385/张</v>
       </c>
       <c r="L60" t="str">
         <v>—</v>
@@ -3577,25 +3109,13 @@
         <v>—</v>
       </c>
       <c r="P60" t="str">
-        <v>ℹ 官方无档 · 价⚠-10.3%</v>
+        <v>ℹ 官方无档 · 价⚠-34.1%</v>
       </c>
       <c r="Q60" t="str">
         <v>Trinity qwen-0925 · 百炼 API qwen-image（统一 ¥0.25/张）</v>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="str">
-        <v/>
-      </c>
-      <c r="B61" t="str">
-        <v/>
-      </c>
-      <c r="C61" t="str">
-        <v/>
-      </c>
-      <c r="D61" t="str">
-        <v/>
-      </c>
       <c r="E61" t="str">
         <v>4K</v>
       </c>
@@ -3615,7 +3135,7 @@
         <v>—</v>
       </c>
       <c r="K61" t="str">
-        <v>$0.063448/张</v>
+        <v>$0.0385/张</v>
       </c>
       <c r="L61" t="str">
         <v>—</v>
@@ -3630,13 +3150,87 @@
         <v>—</v>
       </c>
       <c r="P61" t="str">
-        <v>ℹ 官方无档 · 价⚠-10.3%</v>
+        <v>ℹ 官方无档 · 价⚠-45.6%</v>
       </c>
       <c r="Q61" t="str">
         <v>Trinity qwen-0925 · 百炼 API qwen-image（统一 ¥0.25/张）</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="72">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="B8:B12"/>
+    <mergeCell ref="C8:C12"/>
+    <mergeCell ref="D8:D12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="D13:D15"/>
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="C16:C18"/>
+    <mergeCell ref="D16:D18"/>
+    <mergeCell ref="A19:A21"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="A25:A27"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="D25:D27"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C28:C30"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="A31:A33"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="C31:C33"/>
+    <mergeCell ref="D31:D33"/>
+    <mergeCell ref="A34:A36"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="C34:C36"/>
+    <mergeCell ref="D34:D36"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="C37:C39"/>
+    <mergeCell ref="D37:D39"/>
+    <mergeCell ref="A40:A42"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="D40:D42"/>
+    <mergeCell ref="A43:A46"/>
+    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="C43:C46"/>
+    <mergeCell ref="D43:D46"/>
+    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="C49:C51"/>
+    <mergeCell ref="D49:D51"/>
+    <mergeCell ref="A52:A54"/>
+    <mergeCell ref="B52:B54"/>
+    <mergeCell ref="C52:C54"/>
+    <mergeCell ref="D52:D54"/>
+    <mergeCell ref="A55:A57"/>
+    <mergeCell ref="B55:B57"/>
+    <mergeCell ref="C55:C57"/>
+    <mergeCell ref="D55:D57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="D58:D61"/>
+  </mergeCells>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:Q61"/>
   </ignoredErrors>
@@ -4044,7 +3638,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>生成时间：2026-07-06T10:45:38Z</v>
+        <v>生成时间：2026-07-08T06:32:49Z</v>
       </c>
     </row>
     <row r="24">
@@ -4061,7 +3655,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:J56"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4094,12 +3688,6 @@
       <c r="J1" t="str">
         <v>供应商vs官方</v>
       </c>
-      <c r="K1" t="str">
-        <v>折扣</v>
-      </c>
-      <c r="L1" t="str">
-        <v>成本(元/张)</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -4132,12 +3720,6 @@
       <c r="J2" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K2" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L2" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -4161,12 +3743,6 @@
       <c r="J3" t="str">
         <v>⚠+40%</v>
       </c>
-      <c r="K3" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L3" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -4190,12 +3766,6 @@
       <c r="J4" t="str">
         <v>⚠+80%</v>
       </c>
-      <c r="K4" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L4" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -4228,12 +3798,6 @@
       <c r="J5" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K5" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L5" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -4257,12 +3821,6 @@
       <c r="J6" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K6" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L6" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -4286,12 +3844,6 @@
       <c r="J7" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K7" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L7" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -4324,12 +3876,6 @@
       <c r="J8" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K8" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L8" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -4353,12 +3899,6 @@
       <c r="J9" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K9" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L9" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -4382,12 +3922,6 @@
       <c r="J10" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K10" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L10" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -4420,12 +3954,6 @@
       <c r="J11" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K11" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L11" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -4449,12 +3977,6 @@
       <c r="J12" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K12" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L12" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -4478,12 +4000,6 @@
       <c r="J13" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K13" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L13" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -4516,12 +4032,6 @@
       <c r="J14" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K14" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L14" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -4545,12 +4055,6 @@
       <c r="J15" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K15" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L15" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -4574,12 +4078,6 @@
       <c r="J16" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K16" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L16" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -4612,12 +4110,6 @@
       <c r="J17" t="str">
         <v>⚠+20%</v>
       </c>
-      <c r="K17" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L17" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -4641,12 +4133,6 @@
       <c r="J18" t="str">
         <v>⚠+52%</v>
       </c>
-      <c r="K18" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L18" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -4670,12 +4156,6 @@
       <c r="J19" t="str">
         <v>⚠+84%</v>
       </c>
-      <c r="K19" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L19" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -4708,12 +4188,6 @@
       <c r="J20" t="str">
         <v>—</v>
       </c>
-      <c r="K20" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L20" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -4737,12 +4211,6 @@
       <c r="J21" t="str">
         <v>—</v>
       </c>
-      <c r="K21" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L21" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -4766,12 +4234,6 @@
       <c r="J22" t="str">
         <v>—</v>
       </c>
-      <c r="K22" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L22" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -4804,12 +4266,6 @@
       <c r="J23" t="str">
         <v>—</v>
       </c>
-      <c r="K23" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L23" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -4833,12 +4289,6 @@
       <c r="J24" t="str">
         <v>—</v>
       </c>
-      <c r="K24" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L24" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -4862,12 +4312,6 @@
       <c r="J25" t="str">
         <v>—</v>
       </c>
-      <c r="K25" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L25" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -4900,12 +4344,6 @@
       <c r="J26" t="str">
         <v>—</v>
       </c>
-      <c r="K26" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L26" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -4929,12 +4367,6 @@
       <c r="J27" t="str">
         <v>—</v>
       </c>
-      <c r="K27" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L27" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -4958,12 +4390,6 @@
       <c r="J28" t="str">
         <v>—</v>
       </c>
-      <c r="K28" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L28" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -4996,12 +4422,6 @@
       <c r="J29" t="str">
         <v>—</v>
       </c>
-      <c r="K29" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L29" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -5025,12 +4445,6 @@
       <c r="J30" t="str">
         <v>—</v>
       </c>
-      <c r="K30" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L30" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -5054,12 +4468,6 @@
       <c r="J31" t="str">
         <v>—</v>
       </c>
-      <c r="K31" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L31" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -5092,12 +4500,6 @@
       <c r="J32" t="str">
         <v>—</v>
       </c>
-      <c r="K32" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L32" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -5121,12 +4523,6 @@
       <c r="J33" t="str">
         <v>—</v>
       </c>
-      <c r="K33" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L33" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -5150,12 +4546,6 @@
       <c r="J34" t="str">
         <v>—</v>
       </c>
-      <c r="K34" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L34" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -5188,12 +4578,6 @@
       <c r="J35" t="str">
         <v>—</v>
       </c>
-      <c r="K35" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L35" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -5217,12 +4601,6 @@
       <c r="J36" t="str">
         <v>—</v>
       </c>
-      <c r="K36" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L36" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -5246,12 +4624,6 @@
       <c r="J37" t="str">
         <v>—</v>
       </c>
-      <c r="K37" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L37" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -5284,12 +4656,6 @@
       <c r="J38" t="str">
         <v>—</v>
       </c>
-      <c r="K38" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L38" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -5313,12 +4679,6 @@
       <c r="J39" t="str">
         <v>—</v>
       </c>
-      <c r="K39" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L39" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -5342,12 +4702,6 @@
       <c r="J40" t="str">
         <v>—</v>
       </c>
-      <c r="K40" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L40" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -5371,12 +4725,6 @@
       <c r="J41" t="str">
         <v>—</v>
       </c>
-      <c r="K41" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L41" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -5409,12 +4757,6 @@
       <c r="J42" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K42" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L42" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -5438,12 +4780,6 @@
       <c r="J43" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K43" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L43" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -5467,12 +4803,6 @@
       <c r="J44" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K44" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L44" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -5505,12 +4835,6 @@
       <c r="J45" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K45" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L45" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -5534,12 +4858,6 @@
       <c r="J46" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K46" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L46" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -5563,12 +4881,6 @@
       <c r="J47" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K47" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L47" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -5601,12 +4913,6 @@
       <c r="J48" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K48" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L48" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -5630,12 +4936,6 @@
       <c r="J49" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K49" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L49" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -5659,12 +4959,6 @@
       <c r="J50" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K50" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L50" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -5697,12 +4991,6 @@
       <c r="J51" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K51" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L51" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -5726,12 +5014,6 @@
       <c r="J52" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K52" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L52" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -5755,12 +5037,6 @@
       <c r="J53" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K53" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L53" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -5793,12 +5069,6 @@
       <c r="J54" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K54" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L54" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -5822,12 +5092,6 @@
       <c r="J55" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K55" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L55" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -5850,12 +5114,6 @@
       </c>
       <c r="J56" t="str">
         <v>✅ 一致</v>
-      </c>
-      <c r="K56" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L56" t="str">
-        <v>待填</v>
       </c>
     </row>
   </sheetData>
@@ -5916,14 +5174,14 @@
     <mergeCell ref="D54:D56"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J56"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:J53"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5956,12 +5214,6 @@
       <c r="J1" t="str">
         <v>供应商vs官方</v>
       </c>
-      <c r="K1" t="str">
-        <v>折扣</v>
-      </c>
-      <c r="L1" t="str">
-        <v>成本(美元/张)</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -5994,12 +5246,6 @@
       <c r="J2" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K2" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L2" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -6023,12 +5269,6 @@
       <c r="J3" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K3" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L3" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -6052,12 +5292,6 @@
       <c r="J4" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K4" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L4" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -6090,12 +5324,6 @@
       <c r="J5" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K5" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L5" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -6119,12 +5347,6 @@
       <c r="J6" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K6" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L6" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -6148,12 +5370,6 @@
       <c r="J7" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K7" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L7" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -6186,12 +5402,6 @@
       <c r="J8" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K8" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L8" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -6215,12 +5425,6 @@
       <c r="J9" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K9" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L9" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -6244,12 +5448,6 @@
       <c r="J10" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K10" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L10" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -6282,12 +5480,6 @@
       <c r="J11" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K11" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L11" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -6311,12 +5503,6 @@
       <c r="J12" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K12" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L12" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -6340,12 +5526,6 @@
       <c r="J13" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K13" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L13" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -6378,12 +5558,6 @@
       <c r="J14" t="str">
         <v>⚠+20%</v>
       </c>
-      <c r="K14" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L14" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -6407,12 +5581,6 @@
       <c r="J15" t="str">
         <v>⚠+52%</v>
       </c>
-      <c r="K15" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L15" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -6436,12 +5604,6 @@
       <c r="J16" t="str">
         <v>⚠+84%</v>
       </c>
-      <c r="K16" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L16" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -6474,12 +5636,6 @@
       <c r="J17" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K17" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L17" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -6503,12 +5659,6 @@
       <c r="J18" t="str">
         <v>⚠+30.8%</v>
       </c>
-      <c r="K18" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L18" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -6532,12 +5682,6 @@
       <c r="J19" t="str">
         <v>⚠+61.5%</v>
       </c>
-      <c r="K19" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L19" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -6570,12 +5714,6 @@
       <c r="J20" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K20" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L20" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -6599,12 +5737,6 @@
       <c r="J21" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K21" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L21" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -6628,12 +5760,6 @@
       <c r="J22" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K22" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L22" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -6666,12 +5792,6 @@
       <c r="J23" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K23" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L23" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -6695,12 +5815,6 @@
       <c r="J24" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K24" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L24" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -6724,12 +5838,6 @@
       <c r="J25" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K25" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L25" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -6762,12 +5870,6 @@
       <c r="J26" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K26" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L26" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -6791,12 +5893,6 @@
       <c r="J27" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K27" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L27" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -6820,12 +5916,6 @@
       <c r="J28" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K28" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L28" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -6858,12 +5948,6 @@
       <c r="J29" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K29" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L29" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -6887,12 +5971,6 @@
       <c r="J30" t="str">
         <v>⚠+30.8%</v>
       </c>
-      <c r="K30" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L30" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -6916,12 +5994,6 @@
       <c r="J31" t="str">
         <v>⚠+61.5%</v>
       </c>
-      <c r="K31" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L31" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -6954,12 +6026,6 @@
       <c r="J32" t="str">
         <v>⚠+0.7%</v>
       </c>
-      <c r="K32" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L32" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -6983,12 +6049,6 @@
       <c r="J33" t="str">
         <v>⚠+0.7%</v>
       </c>
-      <c r="K33" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L33" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -7012,12 +6072,6 @@
       <c r="J34" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K34" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L34" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -7050,12 +6104,6 @@
       <c r="J35" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K35" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L35" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -7079,12 +6127,6 @@
       <c r="J36" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K36" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L36" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -7108,12 +6150,6 @@
       <c r="J37" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K37" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L37" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -7137,12 +6173,6 @@
       <c r="J38" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K38" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L38" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -7175,12 +6205,6 @@
       <c r="J39" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K39" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L39" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -7204,12 +6228,6 @@
       <c r="J40" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K40" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L40" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -7233,12 +6251,6 @@
       <c r="J41" t="str">
         <v>✅ 一致</v>
       </c>
-      <c r="K41" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L41" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -7271,12 +6283,6 @@
       <c r="J42" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K42" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L42" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -7300,12 +6306,6 @@
       <c r="J43" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K43" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L43" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -7329,12 +6329,6 @@
       <c r="J44" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K44" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L44" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -7367,12 +6361,6 @@
       <c r="J45" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K45" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L45" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -7396,12 +6384,6 @@
       <c r="J46" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K46" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L46" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -7425,12 +6407,6 @@
       <c r="J47" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K47" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L47" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -7463,12 +6439,6 @@
       <c r="J48" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K48" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L48" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -7492,12 +6462,6 @@
       <c r="J49" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K49" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L49" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -7521,12 +6485,6 @@
       <c r="J50" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K50" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L50" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -7559,12 +6517,6 @@
       <c r="J51" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K51" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L51" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -7588,12 +6540,6 @@
       <c r="J52" t="str">
         <v>⚠-9%</v>
       </c>
-      <c r="K52" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L52" t="str">
-        <v>待填</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -7616,12 +6562,6 @@
       </c>
       <c r="J53" t="str">
         <v>⚠-7.5%</v>
-      </c>
-      <c r="K53" t="str">
-        <v>待填</v>
-      </c>
-      <c r="L53" t="str">
-        <v>待填</v>
       </c>
     </row>
   </sheetData>
@@ -7679,7 +6619,7 @@
     <mergeCell ref="D51:D53"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J53"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>